<commit_message>
more tests on the appended data
</commit_message>
<xml_diff>
--- a/output/PYRQ_output.xlsx
+++ b/output/PYRQ_output.xlsx
@@ -21,6 +21,8 @@
     <sheet name="notes" sheetId="8" state="visible" r:id="rId6"/>
     <sheet name="claim dupes" sheetId="10" state="visible" r:id="rId7"/>
     <sheet name="claim numbers" sheetId="11" state="visible" r:id="rId8"/>
+    <sheet name="closure flag" sheetId="12" state="visible" r:id="rId9"/>
+    <sheet name="closure flag vs case" sheetId="13" state="visible" r:id="rId10"/>
   </sheets>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -123,7 +125,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="16">
+  <numFmts count="33">
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="###0"/>
     <numFmt numFmtId="168" formatCode="###0"/>
@@ -140,6 +142,23 @@
     <numFmt numFmtId="179" formatCode="#,##0"/>
     <numFmt numFmtId="180" formatCode="#,##0"/>
     <numFmt numFmtId="181" formatCode="#,##0"/>
+    <numFmt numFmtId="182" formatCode="#,##0"/>
+    <numFmt numFmtId="183" formatCode="#,##0"/>
+    <numFmt numFmtId="184" formatCode="#,##0"/>
+    <numFmt numFmtId="185" formatCode="#,##0"/>
+    <numFmt numFmtId="186" formatCode="#,##0"/>
+    <numFmt numFmtId="187" formatCode="#,##0"/>
+    <numFmt numFmtId="188" formatCode="#,##0"/>
+    <numFmt numFmtId="189" formatCode="#,##0"/>
+    <numFmt numFmtId="190" formatCode="#,##0"/>
+    <numFmt numFmtId="191" formatCode="#,##0"/>
+    <numFmt numFmtId="192" formatCode="#,##0"/>
+    <numFmt numFmtId="193" formatCode="#,##0"/>
+    <numFmt numFmtId="194" formatCode="#,##0"/>
+    <numFmt numFmtId="195" formatCode="#,##0"/>
+    <numFmt numFmtId="196" formatCode="#,##0"/>
+    <numFmt numFmtId="197" formatCode="#,##0"/>
+    <numFmt numFmtId="198" formatCode="#,##0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -182,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -212,6 +231,36 @@
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="180" xfId="0"/>
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="181" xfId="0"/>
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="181" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="182" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="182" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="183" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="183" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="184" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="184" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="185" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="185" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="186" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="186" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="187" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="187" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="14" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="188" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="189" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="188" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="190" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="191" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="190" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="192" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="193" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="192" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="194" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="195" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="194" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="196" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="197" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="196" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="198" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="198" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -866,6 +915,131 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>closure flag vs case</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be reopen convention, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="58"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="57"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="57"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="57"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="57"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" s="57"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="57"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="57"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B13" s="57"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B14" s="57"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B15" s="57"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B16" s="57"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H11"/>
@@ -3592,4 +3766,101 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>closure flag</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>claim_num</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>acc_date</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>rep_date</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>clsd_date</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>rep_loss</t>
+        </is>
+      </c>
+      <c r="H5" s="38" t="inlineStr">
+        <is>
+          <t>pd_loss</t>
+        </is>
+      </c>
+      <c r="I5" s="38" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="38" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="L5" s="38"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
first pass of error checks
</commit_message>
<xml_diff>
--- a/output/PYRQ_output.xlsx
+++ b/output/PYRQ_output.xlsx
@@ -23,6 +23,16 @@
     <sheet name="claim numbers" sheetId="11" state="visible" r:id="rId8"/>
     <sheet name="closure flag" sheetId="12" state="visible" r:id="rId9"/>
     <sheet name="closure flag vs case" sheetId="13" state="visible" r:id="rId10"/>
+    <sheet name="report date &lt; loss date" sheetId="14" state="visible" r:id="rId11"/>
+    <sheet name="negative paid" sheetId="15" state="visible" r:id="rId12"/>
+    <sheet name="paid+case&lt;&gt;rptd" sheetId="16" state="visible" r:id="rId13"/>
+    <sheet name="paid+case&lt;&gt;rptd" sheetId="17" state="visible" r:id="rId14"/>
+    <sheet name="paid+case&lt;&gt;rptd" sheetId="18" state="visible" r:id="rId15"/>
+    <sheet name="paid+case vs rptd" sheetId="19" state="visible" r:id="rId16"/>
+    <sheet name="paid decreased" sheetId="21" state="visible" r:id="rId17"/>
+    <sheet name="loss or report date changed" sheetId="22" state="visible" r:id="rId18"/>
+    <sheet name="claim number disappeared" sheetId="23" state="visible" r:id="rId19"/>
+    <sheet name="error summary" sheetId="24" state="visible" r:id="rId20"/>
   </sheets>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -125,7 +135,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="33">
+  <numFmts count="73">
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="###0"/>
     <numFmt numFmtId="168" formatCode="###0"/>
@@ -159,6 +169,46 @@
     <numFmt numFmtId="196" formatCode="#,##0"/>
     <numFmt numFmtId="197" formatCode="#,##0"/>
     <numFmt numFmtId="198" formatCode="#,##0"/>
+    <numFmt numFmtId="199" formatCode="#,##0"/>
+    <numFmt numFmtId="200" formatCode="#,##0"/>
+    <numFmt numFmtId="201" formatCode="#,##0"/>
+    <numFmt numFmtId="202" formatCode="#,##0"/>
+    <numFmt numFmtId="203" formatCode="#,##0"/>
+    <numFmt numFmtId="204" formatCode="#,##0"/>
+    <numFmt numFmtId="205" formatCode="#,##0"/>
+    <numFmt numFmtId="206" formatCode="#,##0"/>
+    <numFmt numFmtId="207" formatCode="#,##0"/>
+    <numFmt numFmtId="208" formatCode="#,##0"/>
+    <numFmt numFmtId="209" formatCode="#,##0"/>
+    <numFmt numFmtId="210" formatCode="#,##0"/>
+    <numFmt numFmtId="211" formatCode="#,##0"/>
+    <numFmt numFmtId="212" formatCode="#,##0"/>
+    <numFmt numFmtId="213" formatCode="#,##0"/>
+    <numFmt numFmtId="214" formatCode="#,##0"/>
+    <numFmt numFmtId="215" formatCode="#,##0"/>
+    <numFmt numFmtId="216" formatCode="#,##0"/>
+    <numFmt numFmtId="217" formatCode="#,##0"/>
+    <numFmt numFmtId="218" formatCode="#,##0"/>
+    <numFmt numFmtId="219" formatCode="#,##0"/>
+    <numFmt numFmtId="220" formatCode="#,##0"/>
+    <numFmt numFmtId="221" formatCode="#,##0"/>
+    <numFmt numFmtId="222" formatCode="#,##0"/>
+    <numFmt numFmtId="223" formatCode="#,##0"/>
+    <numFmt numFmtId="224" formatCode="#,##0"/>
+    <numFmt numFmtId="225" formatCode="#,##0"/>
+    <numFmt numFmtId="226" formatCode="#,##0"/>
+    <numFmt numFmtId="227" formatCode="#,##0"/>
+    <numFmt numFmtId="228" formatCode="#,##0"/>
+    <numFmt numFmtId="229" formatCode="#,##0"/>
+    <numFmt numFmtId="230" formatCode="#,##0"/>
+    <numFmt numFmtId="231" formatCode="#,##0"/>
+    <numFmt numFmtId="232" formatCode="#,##0"/>
+    <numFmt numFmtId="233" formatCode="#,##0"/>
+    <numFmt numFmtId="234" formatCode="#,##0"/>
+    <numFmt numFmtId="235" formatCode="#,##0"/>
+    <numFmt numFmtId="236" formatCode="#,##0"/>
+    <numFmt numFmtId="237" formatCode="#,##0"/>
+    <numFmt numFmtId="238" formatCode="#,##0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -201,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -261,6 +311,64 @@
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="196" xfId="0"/>
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="198" xfId="0"/>
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="198" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="199" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="200" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="199" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="201" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="201" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="202" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="203" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="202" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="204" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="205" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="206" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="207" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="208" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="209" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="210" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="211" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="210" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="212" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="213" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="212" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="214" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="215" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="214" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="216" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="217" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="216" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="218" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="219" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="218" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="220" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="221" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="220" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="222" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="223" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="222" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="224" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="225" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="224" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="226" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="227" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="226" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="228" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="229" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="228" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="230" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="231" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="230" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="232" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="233" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="232" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="234" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="235" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="234" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="236" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="237" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="236" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="238" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="238" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1040,6 +1148,3299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:K27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>report date &lt; loss date</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>not sure what could cause this</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>claim_num</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>acc_date</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>rep_date</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr">
+        <is>
+          <t>clsd_date</t>
+        </is>
+      </c>
+      <c r="F5" s="61" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="G5" s="61" t="inlineStr">
+        <is>
+          <t>rep_loss</t>
+        </is>
+      </c>
+      <c r="H5" s="61" t="inlineStr">
+        <is>
+          <t>pd_loss</t>
+        </is>
+      </c>
+      <c r="I5" s="61" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="J5" s="61" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="61"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="59" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C6" s="60">
+        <v>43499</v>
+      </c>
+      <c r="D6" s="60">
+        <v>43617</v>
+      </c>
+      <c r="E6" s="60">
+        <v>44217</v>
+      </c>
+      <c r="F6" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="59">
+        <v>72568</v>
+      </c>
+      <c r="H6" s="59">
+        <v>72568</v>
+      </c>
+      <c r="I6" s="59">
+        <v>0</v>
+      </c>
+      <c r="J6" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="59"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="59" t="inlineStr">
+        <is>
+          <t>A0002</t>
+        </is>
+      </c>
+      <c r="C7" s="60">
+        <v>43629</v>
+      </c>
+      <c r="D7" s="60">
+        <v>44043</v>
+      </c>
+      <c r="E7" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G7" s="59">
+        <v>35287</v>
+      </c>
+      <c r="H7" s="59">
+        <v>27458</v>
+      </c>
+      <c r="I7" s="59">
+        <v>0</v>
+      </c>
+      <c r="J7" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="59"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="59" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C8" s="60">
+        <v>43704</v>
+      </c>
+      <c r="D8" s="60">
+        <v>44109</v>
+      </c>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G8" s="59">
+        <v>86564</v>
+      </c>
+      <c r="H8" s="59">
+        <v>78926</v>
+      </c>
+      <c r="I8" s="59">
+        <v>0</v>
+      </c>
+      <c r="J8" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K8" s="59"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="59" t="inlineStr">
+        <is>
+          <t>A0004</t>
+        </is>
+      </c>
+      <c r="C9" s="60">
+        <v>43721</v>
+      </c>
+      <c r="D9" s="60">
+        <v>44282</v>
+      </c>
+      <c r="E9" s="60">
+        <v>44597</v>
+      </c>
+      <c r="F9" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G9" s="59">
+        <v>7568</v>
+      </c>
+      <c r="H9" s="59">
+        <v>7568</v>
+      </c>
+      <c r="I9" s="59">
+        <v>0</v>
+      </c>
+      <c r="J9" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K9" s="59"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>A0005</t>
+        </is>
+      </c>
+      <c r="C10" s="60">
+        <v>43932</v>
+      </c>
+      <c r="D10" s="60">
+        <v>44489</v>
+      </c>
+      <c r="E10" s="60">
+        <v>44720</v>
+      </c>
+      <c r="F10" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G10" s="59">
+        <v>256845</v>
+      </c>
+      <c r="H10" s="59">
+        <v>256845</v>
+      </c>
+      <c r="I10" s="59">
+        <v>0</v>
+      </c>
+      <c r="J10" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K10" s="59"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="59" t="inlineStr">
+        <is>
+          <t>A0006</t>
+        </is>
+      </c>
+      <c r="C11" s="60">
+        <v>43984</v>
+      </c>
+      <c r="D11" s="60">
+        <v>43994</v>
+      </c>
+      <c r="E11" s="60">
+        <v>44103</v>
+      </c>
+      <c r="F11" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G11" s="59">
+        <v>43718</v>
+      </c>
+      <c r="H11" s="59">
+        <v>43718</v>
+      </c>
+      <c r="I11" s="59">
+        <v>0</v>
+      </c>
+      <c r="J11" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K11" s="59"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" s="59" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="C12" s="60">
+        <v>44064</v>
+      </c>
+      <c r="D12" s="60">
+        <v>44745</v>
+      </c>
+      <c r="E12" s="60">
+        <v>44757</v>
+      </c>
+      <c r="F12" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G12" s="59">
+        <v>7843</v>
+      </c>
+      <c r="H12" s="59">
+        <v>7843</v>
+      </c>
+      <c r="I12" s="59">
+        <v>0</v>
+      </c>
+      <c r="J12" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K12" s="59"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" s="59" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C13" s="60">
+        <v>44203</v>
+      </c>
+      <c r="D13" s="60">
+        <v>44245</v>
+      </c>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F13" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G13" s="59">
+        <v>78300</v>
+      </c>
+      <c r="H13" s="59">
+        <v>23792</v>
+      </c>
+      <c r="I13" s="59">
+        <v>0</v>
+      </c>
+      <c r="J13" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K13" s="59"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" s="59" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C14" s="60">
+        <v>44216</v>
+      </c>
+      <c r="D14" s="60">
+        <v>44325</v>
+      </c>
+      <c r="E14" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F14" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G14" s="59">
+        <v>87824</v>
+      </c>
+      <c r="H14" s="59">
+        <v>79087</v>
+      </c>
+      <c r="I14" s="59">
+        <v>0</v>
+      </c>
+      <c r="J14" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K14" s="59"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" s="59" t="inlineStr">
+        <is>
+          <t>A0011</t>
+        </is>
+      </c>
+      <c r="C15" s="60">
+        <v>44330</v>
+      </c>
+      <c r="D15" s="60">
+        <v>44853</v>
+      </c>
+      <c r="E15" s="60">
+        <v>44897</v>
+      </c>
+      <c r="F15" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G15" s="59">
+        <v>62968</v>
+      </c>
+      <c r="H15" s="59">
+        <v>61968</v>
+      </c>
+      <c r="I15" s="59">
+        <v>0</v>
+      </c>
+      <c r="J15" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K15" s="59"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" s="59" t="inlineStr">
+        <is>
+          <t>A0012</t>
+        </is>
+      </c>
+      <c r="C16" s="60">
+        <v>44302</v>
+      </c>
+      <c r="D16" s="60">
+        <v>44354</v>
+      </c>
+      <c r="E16" s="60">
+        <v>44641</v>
+      </c>
+      <c r="F16" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G16" s="59">
+        <v>44128</v>
+      </c>
+      <c r="H16" s="59">
+        <v>44128</v>
+      </c>
+      <c r="I16" s="59">
+        <v>0</v>
+      </c>
+      <c r="J16" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K16" s="59"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" s="59" t="inlineStr">
+        <is>
+          <t>A0013</t>
+        </is>
+      </c>
+      <c r="C17" s="60">
+        <v>44861</v>
+      </c>
+      <c r="D17" s="60">
+        <v>45011</v>
+      </c>
+      <c r="E17" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F17" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G17" s="59">
+        <v>8399</v>
+      </c>
+      <c r="H17" s="59">
+        <v>6586</v>
+      </c>
+      <c r="I17" s="59">
+        <v>0</v>
+      </c>
+      <c r="J17" s="59" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K17" s="59"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C18" s="60">
+        <v>43499</v>
+      </c>
+      <c r="D18" s="60">
+        <v>43617</v>
+      </c>
+      <c r="E18" s="60">
+        <v>44217</v>
+      </c>
+      <c r="F18" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G18" s="59">
+        <v>74570</v>
+      </c>
+      <c r="H18" s="59">
+        <v>74570</v>
+      </c>
+      <c r="I18" s="59">
+        <v>0</v>
+      </c>
+      <c r="J18" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K18" s="59"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>A0002</t>
+        </is>
+      </c>
+      <c r="C19" s="60">
+        <v>43629</v>
+      </c>
+      <c r="D19" s="60">
+        <v>44043</v>
+      </c>
+      <c r="E19" s="60">
+        <v>44119</v>
+      </c>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G19" s="59">
+        <v>27458</v>
+      </c>
+      <c r="H19" s="59">
+        <v>27458</v>
+      </c>
+      <c r="I19" s="59">
+        <v>0</v>
+      </c>
+      <c r="J19" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K19" s="59"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B20" s="59" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C20" s="60">
+        <v>43704</v>
+      </c>
+      <c r="D20" s="60">
+        <v>44109</v>
+      </c>
+      <c r="E20" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G20" s="59">
+        <v>86564</v>
+      </c>
+      <c r="H20" s="59">
+        <v>77926</v>
+      </c>
+      <c r="I20" s="59">
+        <v>0</v>
+      </c>
+      <c r="J20" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K20" s="59"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B21" s="59" t="inlineStr">
+        <is>
+          <t>A0004</t>
+        </is>
+      </c>
+      <c r="C21" s="60">
+        <v>43721</v>
+      </c>
+      <c r="D21" s="60">
+        <v>44282</v>
+      </c>
+      <c r="E21" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G21" s="59">
+        <v>9811</v>
+      </c>
+      <c r="H21" s="59">
+        <v>5464</v>
+      </c>
+      <c r="I21" s="59">
+        <v>0</v>
+      </c>
+      <c r="J21" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K21" s="59"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B22" s="59" t="inlineStr">
+        <is>
+          <t>A0005</t>
+        </is>
+      </c>
+      <c r="C22" s="60">
+        <v>43932</v>
+      </c>
+      <c r="D22" s="60">
+        <v>44489</v>
+      </c>
+      <c r="E22" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G22" s="59">
+        <v>85426</v>
+      </c>
+      <c r="H22" s="59">
+        <v>18129</v>
+      </c>
+      <c r="I22" s="59">
+        <v>0</v>
+      </c>
+      <c r="J22" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K22" s="59"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B23" s="59" t="inlineStr">
+        <is>
+          <t>A0006</t>
+        </is>
+      </c>
+      <c r="C23" s="60">
+        <v>43984</v>
+      </c>
+      <c r="D23" s="60">
+        <v>43994</v>
+      </c>
+      <c r="E23" s="60">
+        <v>44103</v>
+      </c>
+      <c r="F23" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G23" s="59">
+        <v>43718</v>
+      </c>
+      <c r="H23" s="59">
+        <v>43718</v>
+      </c>
+      <c r="I23" s="59">
+        <v>0</v>
+      </c>
+      <c r="J23" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K23" s="59"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B24" s="59" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="C24" s="60">
+        <v>44054</v>
+      </c>
+      <c r="D24" s="60">
+        <v>44745</v>
+      </c>
+      <c r="E24" s="60">
+        <v>44757</v>
+      </c>
+      <c r="F24" s="59" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G24" s="59">
+        <v>7843</v>
+      </c>
+      <c r="H24" s="59">
+        <v>7843</v>
+      </c>
+      <c r="I24" s="59">
+        <v>0</v>
+      </c>
+      <c r="J24" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K24" s="59"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B25" s="59" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C25" s="60">
+        <v>44203</v>
+      </c>
+      <c r="D25" s="60">
+        <v>44245</v>
+      </c>
+      <c r="E25" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G25" s="59">
+        <v>78300</v>
+      </c>
+      <c r="H25" s="59">
+        <v>25792</v>
+      </c>
+      <c r="I25" s="59">
+        <v>0</v>
+      </c>
+      <c r="J25" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K25" s="59"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B26" s="59" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C26" s="60">
+        <v>44216</v>
+      </c>
+      <c r="D26" s="60">
+        <v>44325</v>
+      </c>
+      <c r="E26" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F26" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G26" s="59">
+        <v>87824</v>
+      </c>
+      <c r="H26" s="59">
+        <v>79087</v>
+      </c>
+      <c r="I26" s="59">
+        <v>0</v>
+      </c>
+      <c r="J26" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K26" s="59"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B27" s="59" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="C27" s="60">
+        <v>44312</v>
+      </c>
+      <c r="D27" s="60">
+        <v>44545</v>
+      </c>
+      <c r="E27" s="60" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F27" s="59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G27" s="59">
+        <v>17378</v>
+      </c>
+      <c r="H27" s="59">
+        <v>12512</v>
+      </c>
+      <c r="I27" s="59">
+        <v>0</v>
+      </c>
+      <c r="J27" s="59" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K27" s="59"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>negative paid</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be recoveries, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="63"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="62"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="62"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="62"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="62"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="62"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="62"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" s="62"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" s="62"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" s="62"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" s="62"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" s="62"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" s="62"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B18" s="62"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B19" s="62"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B20" s="62"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B21" s="62"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B22" s="62"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B23" s="62"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B24" s="62"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B25" s="62"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B26" s="62"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B27" s="62"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>paid+case&lt;&gt;rptd</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be recoveries, expenses, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="70" t="inlineStr">
+        <is>
+          <t>claim_num</t>
+        </is>
+      </c>
+      <c r="C5" s="70" t="inlineStr">
+        <is>
+          <t>acc_date</t>
+        </is>
+      </c>
+      <c r="D5" s="70" t="inlineStr">
+        <is>
+          <t>rep_date</t>
+        </is>
+      </c>
+      <c r="E5" s="70" t="inlineStr">
+        <is>
+          <t>clsd_date</t>
+        </is>
+      </c>
+      <c r="F5" s="70" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="G5" s="70" t="inlineStr">
+        <is>
+          <t>rep_loss</t>
+        </is>
+      </c>
+      <c r="H5" s="70" t="inlineStr">
+        <is>
+          <t>pd_loss</t>
+        </is>
+      </c>
+      <c r="I5" s="70" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="J5" s="70" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="70"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="71" t="inlineStr">
+        <is>
+          <t>A0002</t>
+        </is>
+      </c>
+      <c r="C6" s="72">
+        <v>43629</v>
+      </c>
+      <c r="D6" s="72">
+        <v>44043</v>
+      </c>
+      <c r="E6" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G6" s="71">
+        <v>35287</v>
+      </c>
+      <c r="H6" s="71">
+        <v>27458</v>
+      </c>
+      <c r="I6" s="71">
+        <v>0</v>
+      </c>
+      <c r="J6" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="71"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="71" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C7" s="72">
+        <v>43704</v>
+      </c>
+      <c r="D7" s="72">
+        <v>44109</v>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G7" s="71">
+        <v>86564</v>
+      </c>
+      <c r="H7" s="71">
+        <v>78926</v>
+      </c>
+      <c r="I7" s="71">
+        <v>0</v>
+      </c>
+      <c r="J7" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="71"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B8" s="71" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C8" s="72">
+        <v>44203</v>
+      </c>
+      <c r="D8" s="72">
+        <v>44245</v>
+      </c>
+      <c r="E8" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G8" s="71">
+        <v>78300</v>
+      </c>
+      <c r="H8" s="71">
+        <v>23792</v>
+      </c>
+      <c r="I8" s="71">
+        <v>0</v>
+      </c>
+      <c r="J8" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K8" s="71"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="71" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C9" s="72">
+        <v>44216</v>
+      </c>
+      <c r="D9" s="72">
+        <v>44325</v>
+      </c>
+      <c r="E9" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G9" s="71">
+        <v>87824</v>
+      </c>
+      <c r="H9" s="71">
+        <v>79087</v>
+      </c>
+      <c r="I9" s="71">
+        <v>0</v>
+      </c>
+      <c r="J9" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K9" s="71"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B10" s="71" t="inlineStr">
+        <is>
+          <t>A0011</t>
+        </is>
+      </c>
+      <c r="C10" s="72">
+        <v>44330</v>
+      </c>
+      <c r="D10" s="72">
+        <v>44853</v>
+      </c>
+      <c r="E10" s="72">
+        <v>44897</v>
+      </c>
+      <c r="F10" s="71" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G10" s="71">
+        <v>62968</v>
+      </c>
+      <c r="H10" s="71">
+        <v>61968</v>
+      </c>
+      <c r="I10" s="71">
+        <v>0</v>
+      </c>
+      <c r="J10" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K10" s="71"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>A0013</t>
+        </is>
+      </c>
+      <c r="C11" s="72">
+        <v>44861</v>
+      </c>
+      <c r="D11" s="72">
+        <v>45011</v>
+      </c>
+      <c r="E11" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G11" s="71">
+        <v>8399</v>
+      </c>
+      <c r="H11" s="71">
+        <v>6586</v>
+      </c>
+      <c r="I11" s="71">
+        <v>0</v>
+      </c>
+      <c r="J11" s="71" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K11" s="71"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B12" s="71" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C12" s="72">
+        <v>43704</v>
+      </c>
+      <c r="D12" s="72">
+        <v>44109</v>
+      </c>
+      <c r="E12" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F12" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G12" s="71">
+        <v>86564</v>
+      </c>
+      <c r="H12" s="71">
+        <v>77926</v>
+      </c>
+      <c r="I12" s="71">
+        <v>0</v>
+      </c>
+      <c r="J12" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K12" s="71"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B13" s="71" t="inlineStr">
+        <is>
+          <t>A0004</t>
+        </is>
+      </c>
+      <c r="C13" s="72">
+        <v>43721</v>
+      </c>
+      <c r="D13" s="72">
+        <v>44282</v>
+      </c>
+      <c r="E13" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F13" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G13" s="71">
+        <v>9811</v>
+      </c>
+      <c r="H13" s="71">
+        <v>5464</v>
+      </c>
+      <c r="I13" s="71">
+        <v>0</v>
+      </c>
+      <c r="J13" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K13" s="71"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="inlineStr">
+        <is>
+          <t>A0005</t>
+        </is>
+      </c>
+      <c r="C14" s="72">
+        <v>43932</v>
+      </c>
+      <c r="D14" s="72">
+        <v>44489</v>
+      </c>
+      <c r="E14" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F14" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G14" s="71">
+        <v>85426</v>
+      </c>
+      <c r="H14" s="71">
+        <v>18129</v>
+      </c>
+      <c r="I14" s="71">
+        <v>0</v>
+      </c>
+      <c r="J14" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K14" s="71"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B15" s="71" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C15" s="72">
+        <v>44203</v>
+      </c>
+      <c r="D15" s="72">
+        <v>44245</v>
+      </c>
+      <c r="E15" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F15" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G15" s="71">
+        <v>78300</v>
+      </c>
+      <c r="H15" s="71">
+        <v>25792</v>
+      </c>
+      <c r="I15" s="71">
+        <v>0</v>
+      </c>
+      <c r="J15" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K15" s="71"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B16" s="71" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C16" s="72">
+        <v>44216</v>
+      </c>
+      <c r="D16" s="72">
+        <v>44325</v>
+      </c>
+      <c r="E16" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F16" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G16" s="71">
+        <v>87824</v>
+      </c>
+      <c r="H16" s="71">
+        <v>79087</v>
+      </c>
+      <c r="I16" s="71">
+        <v>0</v>
+      </c>
+      <c r="J16" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K16" s="71"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B17" s="71" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="C17" s="72">
+        <v>44312</v>
+      </c>
+      <c r="D17" s="72">
+        <v>44545</v>
+      </c>
+      <c r="E17" s="72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F17" s="71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G17" s="71">
+        <v>17378</v>
+      </c>
+      <c r="H17" s="71">
+        <v>12512</v>
+      </c>
+      <c r="I17" s="71">
+        <v>0</v>
+      </c>
+      <c r="J17" s="71" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="K17" s="71"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be recoveries, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="90" t="inlineStr">
+        <is>
+          <t>claim_num.c</t>
+        </is>
+      </c>
+      <c r="C5" s="90" t="inlineStr">
+        <is>
+          <t>acc_date.c</t>
+        </is>
+      </c>
+      <c r="D5" s="90" t="inlineStr">
+        <is>
+          <t>rep_date.c</t>
+        </is>
+      </c>
+      <c r="E5" s="90" t="inlineStr">
+        <is>
+          <t>clsd_date.c</t>
+        </is>
+      </c>
+      <c r="F5" s="90" t="inlineStr">
+        <is>
+          <t>claim_status.c</t>
+        </is>
+      </c>
+      <c r="G5" s="90" t="inlineStr">
+        <is>
+          <t>rep_loss.c</t>
+        </is>
+      </c>
+      <c r="H5" s="90" t="inlineStr">
+        <is>
+          <t>pd_loss.c</t>
+        </is>
+      </c>
+      <c r="I5" s="90" t="inlineStr">
+        <is>
+          <t>case_loss.c</t>
+        </is>
+      </c>
+      <c r="J5" s="90" t="inlineStr">
+        <is>
+          <t>source.c</t>
+        </is>
+      </c>
+      <c r="K5" s="90" t="inlineStr">
+        <is>
+          <t>claim_num.p</t>
+        </is>
+      </c>
+      <c r="L5" s="90" t="inlineStr">
+        <is>
+          <t>acc_date.p</t>
+        </is>
+      </c>
+      <c r="M5" s="90" t="inlineStr">
+        <is>
+          <t>rep_date.p</t>
+        </is>
+      </c>
+      <c r="N5" s="90" t="inlineStr">
+        <is>
+          <t>clsd_date.p</t>
+        </is>
+      </c>
+      <c r="O5" s="90" t="inlineStr">
+        <is>
+          <t>claim_status.p</t>
+        </is>
+      </c>
+      <c r="P5" s="90" t="inlineStr">
+        <is>
+          <t>rep_loss.p</t>
+        </is>
+      </c>
+      <c r="Q5" s="90" t="inlineStr">
+        <is>
+          <t>pd_loss.p</t>
+        </is>
+      </c>
+      <c r="R5" s="90" t="inlineStr">
+        <is>
+          <t>case_loss.p</t>
+        </is>
+      </c>
+      <c r="S5" s="90" t="inlineStr">
+        <is>
+          <t>source.p</t>
+        </is>
+      </c>
+      <c r="T5" s="90"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="88" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C6" s="89">
+        <v>43499</v>
+      </c>
+      <c r="D6" s="89">
+        <v>43617</v>
+      </c>
+      <c r="E6" s="89">
+        <v>44217</v>
+      </c>
+      <c r="F6" s="88" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="88">
+        <v>72568</v>
+      </c>
+      <c r="H6" s="88">
+        <v>72568</v>
+      </c>
+      <c r="I6" s="88">
+        <v>0</v>
+      </c>
+      <c r="J6" s="88" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="88" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="L6" s="89">
+        <v>43499</v>
+      </c>
+      <c r="M6" s="89">
+        <v>43617</v>
+      </c>
+      <c r="N6" s="89">
+        <v>44217</v>
+      </c>
+      <c r="O6" s="88" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P6" s="88">
+        <v>74570</v>
+      </c>
+      <c r="Q6" s="88">
+        <v>74570</v>
+      </c>
+      <c r="R6" s="88">
+        <v>0</v>
+      </c>
+      <c r="S6" s="88" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="88"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B7" s="88" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C7" s="89">
+        <v>44203</v>
+      </c>
+      <c r="D7" s="89">
+        <v>44245</v>
+      </c>
+      <c r="E7" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="88" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G7" s="88">
+        <v>78300</v>
+      </c>
+      <c r="H7" s="88">
+        <v>23792</v>
+      </c>
+      <c r="I7" s="88">
+        <v>54508</v>
+      </c>
+      <c r="J7" s="88" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="88" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="L7" s="89">
+        <v>44203</v>
+      </c>
+      <c r="M7" s="89">
+        <v>44245</v>
+      </c>
+      <c r="N7" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="88" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P7" s="88">
+        <v>78300</v>
+      </c>
+      <c r="Q7" s="88">
+        <v>25792</v>
+      </c>
+      <c r="R7" s="88">
+        <v>52508</v>
+      </c>
+      <c r="S7" s="88" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T7" s="88"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="B8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S8" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" s="88"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>NA.1</t>
+        </is>
+      </c>
+      <c r="B9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S9" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" s="88"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>NA.2</t>
+        </is>
+      </c>
+      <c r="B10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N10" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S10" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T10" s="88"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>NA.3</t>
+        </is>
+      </c>
+      <c r="B11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N11" s="89" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S11" s="88" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T11" s="88"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be recoveries, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="108" t="inlineStr">
+        <is>
+          <t>claim_num.c</t>
+        </is>
+      </c>
+      <c r="C5" s="108" t="inlineStr">
+        <is>
+          <t>acc_date.c</t>
+        </is>
+      </c>
+      <c r="D5" s="108" t="inlineStr">
+        <is>
+          <t>rep_date.c</t>
+        </is>
+      </c>
+      <c r="E5" s="108" t="inlineStr">
+        <is>
+          <t>clsd_date.c</t>
+        </is>
+      </c>
+      <c r="F5" s="108" t="inlineStr">
+        <is>
+          <t>claim_status.c</t>
+        </is>
+      </c>
+      <c r="G5" s="108" t="inlineStr">
+        <is>
+          <t>rep_loss.c</t>
+        </is>
+      </c>
+      <c r="H5" s="108" t="inlineStr">
+        <is>
+          <t>pd_loss.c</t>
+        </is>
+      </c>
+      <c r="I5" s="108" t="inlineStr">
+        <is>
+          <t>case_loss.c</t>
+        </is>
+      </c>
+      <c r="J5" s="108" t="inlineStr">
+        <is>
+          <t>source.c</t>
+        </is>
+      </c>
+      <c r="K5" s="108" t="inlineStr">
+        <is>
+          <t>claim_num.p</t>
+        </is>
+      </c>
+      <c r="L5" s="108" t="inlineStr">
+        <is>
+          <t>acc_date.p</t>
+        </is>
+      </c>
+      <c r="M5" s="108" t="inlineStr">
+        <is>
+          <t>rep_date.p</t>
+        </is>
+      </c>
+      <c r="N5" s="108" t="inlineStr">
+        <is>
+          <t>clsd_date.p</t>
+        </is>
+      </c>
+      <c r="O5" s="108" t="inlineStr">
+        <is>
+          <t>claim_status.p</t>
+        </is>
+      </c>
+      <c r="P5" s="108" t="inlineStr">
+        <is>
+          <t>rep_loss.p</t>
+        </is>
+      </c>
+      <c r="Q5" s="108" t="inlineStr">
+        <is>
+          <t>pd_loss.p</t>
+        </is>
+      </c>
+      <c r="R5" s="108" t="inlineStr">
+        <is>
+          <t>case_loss.p</t>
+        </is>
+      </c>
+      <c r="S5" s="108" t="inlineStr">
+        <is>
+          <t>source.p</t>
+        </is>
+      </c>
+      <c r="T5" s="108"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="106" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C6" s="107">
+        <v>43499</v>
+      </c>
+      <c r="D6" s="107">
+        <v>43617</v>
+      </c>
+      <c r="E6" s="107">
+        <v>44217</v>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="106">
+        <v>72568</v>
+      </c>
+      <c r="H6" s="106">
+        <v>72568</v>
+      </c>
+      <c r="I6" s="106">
+        <v>0</v>
+      </c>
+      <c r="J6" s="106" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="106" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="L6" s="107">
+        <v>43499</v>
+      </c>
+      <c r="M6" s="107">
+        <v>43617</v>
+      </c>
+      <c r="N6" s="107">
+        <v>44217</v>
+      </c>
+      <c r="O6" s="106" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P6" s="106">
+        <v>74570</v>
+      </c>
+      <c r="Q6" s="106">
+        <v>74570</v>
+      </c>
+      <c r="R6" s="106">
+        <v>0</v>
+      </c>
+      <c r="S6" s="106" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="106"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B7" s="106" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C7" s="107">
+        <v>44203</v>
+      </c>
+      <c r="D7" s="107">
+        <v>44245</v>
+      </c>
+      <c r="E7" s="107" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="106" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G7" s="106">
+        <v>78300</v>
+      </c>
+      <c r="H7" s="106">
+        <v>23792</v>
+      </c>
+      <c r="I7" s="106">
+        <v>54508</v>
+      </c>
+      <c r="J7" s="106" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="106" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="L7" s="107">
+        <v>44203</v>
+      </c>
+      <c r="M7" s="107">
+        <v>44245</v>
+      </c>
+      <c r="N7" s="107" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="106" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P7" s="106">
+        <v>78300</v>
+      </c>
+      <c r="Q7" s="106">
+        <v>25792</v>
+      </c>
+      <c r="R7" s="106">
+        <v>52508</v>
+      </c>
+      <c r="S7" s="106" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T7" s="106"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be error correction, reopen, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="111" t="inlineStr">
+        <is>
+          <t>claim_num.c</t>
+        </is>
+      </c>
+      <c r="C5" s="111" t="inlineStr">
+        <is>
+          <t>acc_date.c</t>
+        </is>
+      </c>
+      <c r="D5" s="111" t="inlineStr">
+        <is>
+          <t>rep_date.c</t>
+        </is>
+      </c>
+      <c r="E5" s="111" t="inlineStr">
+        <is>
+          <t>clsd_date.c</t>
+        </is>
+      </c>
+      <c r="F5" s="111" t="inlineStr">
+        <is>
+          <t>claim_status.c</t>
+        </is>
+      </c>
+      <c r="G5" s="111" t="inlineStr">
+        <is>
+          <t>rep_loss.c</t>
+        </is>
+      </c>
+      <c r="H5" s="111" t="inlineStr">
+        <is>
+          <t>pd_loss.c</t>
+        </is>
+      </c>
+      <c r="I5" s="111" t="inlineStr">
+        <is>
+          <t>case_loss.c</t>
+        </is>
+      </c>
+      <c r="J5" s="111" t="inlineStr">
+        <is>
+          <t>source.c</t>
+        </is>
+      </c>
+      <c r="K5" s="111" t="inlineStr">
+        <is>
+          <t>claim_num.p</t>
+        </is>
+      </c>
+      <c r="L5" s="111" t="inlineStr">
+        <is>
+          <t>acc_date.p</t>
+        </is>
+      </c>
+      <c r="M5" s="111" t="inlineStr">
+        <is>
+          <t>rep_date.p</t>
+        </is>
+      </c>
+      <c r="N5" s="111" t="inlineStr">
+        <is>
+          <t>clsd_date.p</t>
+        </is>
+      </c>
+      <c r="O5" s="111" t="inlineStr">
+        <is>
+          <t>claim_status.p</t>
+        </is>
+      </c>
+      <c r="P5" s="111" t="inlineStr">
+        <is>
+          <t>rep_loss.p</t>
+        </is>
+      </c>
+      <c r="Q5" s="111" t="inlineStr">
+        <is>
+          <t>pd_loss.p</t>
+        </is>
+      </c>
+      <c r="R5" s="111" t="inlineStr">
+        <is>
+          <t>case_loss.p</t>
+        </is>
+      </c>
+      <c r="S5" s="111" t="inlineStr">
+        <is>
+          <t>source.p</t>
+        </is>
+      </c>
+      <c r="T5" s="111"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" s="109" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="C6" s="110">
+        <v>44064</v>
+      </c>
+      <c r="D6" s="110">
+        <v>44745</v>
+      </c>
+      <c r="E6" s="110">
+        <v>44757</v>
+      </c>
+      <c r="F6" s="109" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="109">
+        <v>7843</v>
+      </c>
+      <c r="H6" s="109">
+        <v>7843</v>
+      </c>
+      <c r="I6" s="109">
+        <v>0</v>
+      </c>
+      <c r="J6" s="109" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="109" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="L6" s="110">
+        <v>44054</v>
+      </c>
+      <c r="M6" s="110">
+        <v>44745</v>
+      </c>
+      <c r="N6" s="110">
+        <v>44757</v>
+      </c>
+      <c r="O6" s="109" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P6" s="109">
+        <v>7843</v>
+      </c>
+      <c r="Q6" s="109">
+        <v>7843</v>
+      </c>
+      <c r="R6" s="109">
+        <v>0</v>
+      </c>
+      <c r="S6" s="109" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="109"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="114" t="inlineStr">
+        <is>
+          <t>claim_num.current</t>
+        </is>
+      </c>
+      <c r="C5" s="114" t="inlineStr">
+        <is>
+          <t>.currentc_date.c</t>
+        </is>
+      </c>
+      <c r="D5" s="114" t="inlineStr">
+        <is>
+          <t>r.prior_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="114" t="inlineStr">
+        <is>
+          <t>clsd_date.current</t>
+        </is>
+      </c>
+      <c r="F5" s="114" t="inlineStr">
+        <is>
+          <t>claim_status.current</t>
+        </is>
+      </c>
+      <c r="G5" s="114" t="inlineStr">
+        <is>
+          <t>r.prior_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="114" t="inlineStr">
+        <is>
+          <t>pd_loss.current</t>
+        </is>
+      </c>
+      <c r="I5" s="114" t="inlineStr">
+        <is>
+          <t>case_loss.current</t>
+        </is>
+      </c>
+      <c r="J5" s="114" t="inlineStr">
+        <is>
+          <t>sou.currente.c</t>
+        </is>
+      </c>
+      <c r="K5" s="114" t="inlineStr">
+        <is>
+          <t>claim_num.prior</t>
+        </is>
+      </c>
+      <c r="L5" s="114" t="inlineStr">
+        <is>
+          <t>.currentc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="114" t="inlineStr">
+        <is>
+          <t>r.prior_date.p</t>
+        </is>
+      </c>
+      <c r="N5" s="114" t="inlineStr">
+        <is>
+          <t>clsd_date.prior</t>
+        </is>
+      </c>
+      <c r="O5" s="114" t="inlineStr">
+        <is>
+          <t>claim_status.prior</t>
+        </is>
+      </c>
+      <c r="P5" s="114" t="inlineStr">
+        <is>
+          <t>r.prior_loss.p</t>
+        </is>
+      </c>
+      <c r="Q5" s="114" t="inlineStr">
+        <is>
+          <t>pd_loss.prior</t>
+        </is>
+      </c>
+      <c r="R5" s="114" t="inlineStr">
+        <is>
+          <t>case_loss.prior</t>
+        </is>
+      </c>
+      <c r="S5" s="114" t="inlineStr">
+        <is>
+          <t>sou.currente.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="114"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6" s="113" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D6" s="113" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E6" s="113" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" s="112" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K6" s="112" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="L6" s="113">
+        <v>44312</v>
+      </c>
+      <c r="M6" s="113">
+        <v>44545</v>
+      </c>
+      <c r="N6" s="113" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="112" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P6" s="112">
+        <v>17378</v>
+      </c>
+      <c r="Q6" s="112">
+        <v>12512</v>
+      </c>
+      <c r="R6" s="112">
+        <v>4866</v>
+      </c>
+      <c r="S6" s="112" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="112"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H11"/>
@@ -1326,6 +4727,313 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFFFC0CB"/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>error summary</t>
+        </is>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>table of error types and counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="116" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C5" s="116" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D5" s="116" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E5" s="116"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="115" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="C6" s="115" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="D6" s="115">
+        <v>1</v>
+      </c>
+      <c r="E6" s="115"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="115" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="C7" s="115" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="D7" s="115">
+        <v>6</v>
+      </c>
+      <c r="E7" s="115"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="C8" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="D8" s="115">
+        <v>5</v>
+      </c>
+      <c r="E8" s="115"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="C9" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="D9" s="115">
+        <v>5</v>
+      </c>
+      <c r="E9" s="115"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="C10" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="D10" s="115">
+        <v>5</v>
+      </c>
+      <c r="E10" s="115"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="C11" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="D11" s="115">
+        <v>6</v>
+      </c>
+      <c r="E11" s="115"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="C12" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="D12" s="115">
+        <v>9</v>
+      </c>
+      <c r="E12" s="115"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="C13" s="115" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="D13" s="115">
+        <v>2</v>
+      </c>
+      <c r="E13" s="115"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="C14" s="115" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="D14" s="115">
+        <v>1</v>
+      </c>
+      <c r="E14" s="115"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" s="115" t="inlineStr">
+        <is>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="C15" s="115" t="inlineStr">
+        <is>
+          <t>claim number present in prior but not current</t>
+        </is>
+      </c>
+      <c r="D15" s="115">
+        <v>0</v>
+      </c>
+      <c r="E15" s="115"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" s="115" t="inlineStr">
+        <is>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="C16" s="115" t="inlineStr">
+        <is>
+          <t>claim number present in prior but not current</t>
+        </is>
+      </c>
+      <c r="D16" s="115">
+        <v>0</v>
+      </c>
+      <c r="E16" s="115"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" s="115" t="inlineStr">
+        <is>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="C17" s="115" t="inlineStr">
+        <is>
+          <t>claim number present in prior but not current</t>
+        </is>
+      </c>
+      <c r="D17" s="115">
+        <v>1</v>
+      </c>
+      <c r="E17" s="115"/>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
report date test WIP
</commit_message>
<xml_diff>
--- a/output/PYRQ_output.xlsx
+++ b/output/PYRQ_output.xlsx
@@ -19,13 +19,13 @@
     <sheet name="initial diagnostics" sheetId="6" state="visible" r:id="rId4"/>
     <sheet name="triangles" sheetId="7" state="visible" r:id="rId5"/>
     <sheet name="notes" sheetId="8" state="visible" r:id="rId6"/>
-    <sheet name="claim numbers" sheetId="31" state="visible" r:id="rId7"/>
-    <sheet name="closure flag vs case" sheetId="32" state="visible" r:id="rId8"/>
-    <sheet name="paid+case vs rptd" sheetId="33" state="visible" r:id="rId9"/>
-    <sheet name="paid decreased" sheetId="34" state="visible" r:id="rId10"/>
-    <sheet name="loss or report date changed" sheetId="35" state="visible" r:id="rId11"/>
-    <sheet name="claim number disappeared" sheetId="36" state="visible" r:id="rId12"/>
-    <sheet name="error summary" sheetId="37" state="visible" r:id="rId13"/>
+    <sheet name="error summary" sheetId="37" state="visible" r:id="rId7"/>
+    <sheet name="claim numbers" sheetId="38" state="visible" r:id="rId8"/>
+    <sheet name="closure flag vs case" sheetId="39" state="visible" r:id="rId9"/>
+    <sheet name="paid+case vs rptd" sheetId="40" state="visible" r:id="rId10"/>
+    <sheet name="paid decreased" sheetId="41" state="visible" r:id="rId11"/>
+    <sheet name="loss or report date changed" sheetId="42" state="visible" r:id="rId12"/>
+    <sheet name="claim number disappeared" sheetId="43" state="visible" r:id="rId13"/>
   </sheets>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -128,7 +128,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="166">
+  <numFmts count="213">
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="###0"/>
     <numFmt numFmtId="168" formatCode="###0"/>
@@ -295,6 +295,53 @@
     <numFmt numFmtId="329" formatCode="YYYY\/MM\/DD"/>
     <numFmt numFmtId="330" formatCode="YYYY\/MM\/DD"/>
     <numFmt numFmtId="331" formatCode="#,##0"/>
+    <numFmt numFmtId="332" formatCode="#,##0"/>
+    <numFmt numFmtId="333" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="334" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="335" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="336" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="337" formatCode="#,##0"/>
+    <numFmt numFmtId="338" formatCode="#,##0"/>
+    <numFmt numFmtId="339" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="340" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="341" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="342" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="343" formatCode="#,##0"/>
+    <numFmt numFmtId="344" formatCode="#,##0"/>
+    <numFmt numFmtId="345" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="346" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="347" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="348" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="349" formatCode="#,##0"/>
+    <numFmt numFmtId="350" formatCode="#,##0"/>
+    <numFmt numFmtId="351" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="352" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="353" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="354" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="355" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="356" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="357" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="358" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="359" formatCode="#,##0"/>
+    <numFmt numFmtId="360" formatCode="#,##0"/>
+    <numFmt numFmtId="361" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="362" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="363" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="364" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="365" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="366" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="367" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="368" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="369" formatCode="#,##0"/>
+    <numFmt numFmtId="370" formatCode="#,##0"/>
+    <numFmt numFmtId="371" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="372" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="373" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="374" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="375" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="376" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="377" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="378" formatCode="YYYY\/MM\/DD"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -337,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="203">
+  <cellXfs count="256">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -541,6 +588,59 @@
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="330" xfId="0"/>
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="331" xfId="0"/>
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="331" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="332" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="332" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="333" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="334" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="335" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="336" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="337" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="338" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="337" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="339" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="340" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="341" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="342" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="343" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="344" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="343" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="345" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="346" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="347" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="348" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="349" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="350" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="349" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="351" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="352" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="353" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="354" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="355" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="356" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="357" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="358" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="359" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="360" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="359" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="361" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="362" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="363" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="364" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="365" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="366" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="367" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="368" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="369" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="370" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="369" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="371" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="372" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="373" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="374" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="375" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="376" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="377" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="378" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1200,328 +1300,150 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="11" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>paid decreased</t>
+          <t>paid+case vs rptd</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
-      <c r="E1" s="171"/>
+      <c r="C1" s="219"/>
+      <c r="D1" s="219"/>
+      <c r="E1" s="219"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
-      <c r="L1" s="175"/>
-      <c r="M1" s="175"/>
-      <c r="N1" s="175"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be recoveries, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="172"/>
-      <c r="D2" s="172"/>
-      <c r="E2" s="172"/>
-      <c r="L2" s="176"/>
-      <c r="M2" s="176"/>
-      <c r="N2" s="176"/>
+          <t>could be recoveries, expenses, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="220"/>
+      <c r="D2" s="220"/>
+      <c r="E2" s="220"/>
     </row>
     <row r="3">
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="L3" s="176"/>
-      <c r="M3" s="176"/>
-      <c r="N3" s="176"/>
+      <c r="C3" s="220"/>
+      <c r="D3" s="220"/>
+      <c r="E3" s="220"/>
     </row>
     <row r="4">
-      <c r="C4" s="172"/>
-      <c r="D4" s="172"/>
-      <c r="E4" s="172"/>
-      <c r="L4" s="176"/>
-      <c r="M4" s="176"/>
-      <c r="N4" s="176"/>
+      <c r="C4" s="220"/>
+      <c r="D4" s="220"/>
+      <c r="E4" s="220"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="170" t="inlineStr">
-        <is>
-          <t>claim_num.current</t>
-        </is>
-      </c>
-      <c r="C5" s="173" t="inlineStr">
-        <is>
-          <t>.currentc_date.c</t>
-        </is>
-      </c>
-      <c r="D5" s="173" t="inlineStr">
-        <is>
-          <t>r.prior_date.current</t>
-        </is>
-      </c>
-      <c r="E5" s="173" t="inlineStr">
-        <is>
-          <t>clsd_date.current</t>
-        </is>
-      </c>
-      <c r="F5" s="170" t="inlineStr">
-        <is>
-          <t>claim_status.current</t>
-        </is>
-      </c>
-      <c r="G5" s="170" t="inlineStr">
-        <is>
-          <t>r.prior_loss.current</t>
-        </is>
-      </c>
-      <c r="H5" s="170" t="inlineStr">
-        <is>
-          <t>pd_loss.current</t>
-        </is>
-      </c>
-      <c r="I5" s="170" t="inlineStr">
-        <is>
-          <t>case_loss.current</t>
-        </is>
-      </c>
-      <c r="J5" s="170" t="inlineStr">
-        <is>
-          <t>sou.currente.c</t>
-        </is>
-      </c>
-      <c r="K5" s="170" t="inlineStr">
-        <is>
-          <t>claim_num.prior</t>
-        </is>
-      </c>
-      <c r="L5" s="177" t="inlineStr">
-        <is>
-          <t>.currentc_date.prior</t>
-        </is>
-      </c>
-      <c r="M5" s="177" t="inlineStr">
-        <is>
-          <t>r.prior_date.p</t>
-        </is>
-      </c>
-      <c r="N5" s="177" t="inlineStr">
-        <is>
-          <t>clsd_date.prior</t>
-        </is>
-      </c>
-      <c r="O5" s="170" t="inlineStr">
-        <is>
-          <t>claim_status.prior</t>
-        </is>
-      </c>
-      <c r="P5" s="170" t="inlineStr">
-        <is>
-          <t>r.prior_loss.p</t>
-        </is>
-      </c>
-      <c r="Q5" s="170" t="inlineStr">
-        <is>
-          <t>pd_loss.prior</t>
-        </is>
-      </c>
-      <c r="R5" s="170" t="inlineStr">
-        <is>
-          <t>case_loss.prior</t>
-        </is>
-      </c>
-      <c r="S5" s="170" t="inlineStr">
-        <is>
-          <t>sou.currente.prior</t>
-        </is>
-      </c>
-      <c r="T5" s="170"/>
+      <c r="B5" s="218" t="inlineStr">
+        <is>
+          <t>claim_num</t>
+        </is>
+      </c>
+      <c r="C5" s="221" t="inlineStr">
+        <is>
+          <t>acc_date</t>
+        </is>
+      </c>
+      <c r="D5" s="221" t="inlineStr">
+        <is>
+          <t>rep_date</t>
+        </is>
+      </c>
+      <c r="E5" s="221" t="inlineStr">
+        <is>
+          <t>clsd_date</t>
+        </is>
+      </c>
+      <c r="F5" s="218" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="G5" s="218" t="inlineStr">
+        <is>
+          <t>rep_loss</t>
+        </is>
+      </c>
+      <c r="H5" s="218" t="inlineStr">
+        <is>
+          <t>pd_loss</t>
+        </is>
+      </c>
+      <c r="I5" s="218" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="J5" s="218" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="218"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="168" t="inlineStr">
-        <is>
-          <t>A0001</t>
-        </is>
-      </c>
-      <c r="C6" s="174">
-        <v>43499</v>
-      </c>
-      <c r="D6" s="174">
-        <v>43617</v>
-      </c>
-      <c r="E6" s="174">
-        <v>44217</v>
-      </c>
-      <c r="F6" s="168" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="G6" s="168">
-        <v>72568</v>
-      </c>
-      <c r="H6" s="168">
-        <v>72568</v>
-      </c>
-      <c r="I6" s="168">
-        <v>0</v>
-      </c>
-      <c r="J6" s="168" t="inlineStr">
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="216" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C6" s="222">
+        <v>43704</v>
+      </c>
+      <c r="D6" s="222">
+        <v>44109</v>
+      </c>
+      <c r="E6" s="222" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="216" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G6" s="216">
+        <v>86564</v>
+      </c>
+      <c r="H6" s="216">
+        <v>78926</v>
+      </c>
+      <c r="I6" s="216">
+        <v>8638</v>
+      </c>
+      <c r="J6" s="216" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="168" t="inlineStr">
-        <is>
-          <t>A0001</t>
-        </is>
-      </c>
-      <c r="L6" s="178">
-        <v>43499</v>
-      </c>
-      <c r="M6" s="178">
-        <v>43617</v>
-      </c>
-      <c r="N6" s="178">
-        <v>44217</v>
-      </c>
-      <c r="O6" s="168" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="P6" s="168">
-        <v>74570</v>
-      </c>
-      <c r="Q6" s="168">
-        <v>74570</v>
-      </c>
-      <c r="R6" s="168">
-        <v>0</v>
-      </c>
-      <c r="S6" s="168" t="inlineStr">
-        <is>
-          <t>ex1_prior</t>
-        </is>
-      </c>
-      <c r="T6" s="168"/>
+      <c r="K6" s="216"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B7" s="168" t="inlineStr">
-        <is>
-          <t>A0008</t>
-        </is>
-      </c>
-      <c r="C7" s="174">
-        <v>44203</v>
-      </c>
-      <c r="D7" s="174">
-        <v>44245</v>
-      </c>
-      <c r="E7" s="174" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" s="168" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G7" s="168">
-        <v>78300</v>
-      </c>
-      <c r="H7" s="168">
-        <v>23792</v>
-      </c>
-      <c r="I7" s="168">
-        <v>54508</v>
-      </c>
-      <c r="J7" s="168" t="inlineStr">
-        <is>
-          <t>ex1_curr</t>
-        </is>
-      </c>
-      <c r="K7" s="168" t="inlineStr">
-        <is>
-          <t>A0008</t>
-        </is>
-      </c>
-      <c r="L7" s="178">
-        <v>44203</v>
-      </c>
-      <c r="M7" s="178">
-        <v>44245</v>
-      </c>
-      <c r="N7" s="178" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O7" s="168" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="P7" s="168">
-        <v>78300</v>
-      </c>
-      <c r="Q7" s="168">
-        <v>25792</v>
-      </c>
-      <c r="R7" s="168">
-        <v>52508</v>
-      </c>
-      <c r="S7" s="168" t="inlineStr">
-        <is>
-          <t>ex1_prior</t>
-        </is>
-      </c>
-      <c r="T7" s="168"/>
+      <c r="C7" s="220"/>
+      <c r="D7" s="220"/>
+      <c r="E7" s="220"/>
     </row>
     <row r="8">
-      <c r="C8" s="172"/>
-      <c r="D8" s="172"/>
-      <c r="E8" s="172"/>
-      <c r="L8" s="176"/>
-      <c r="M8" s="176"/>
-      <c r="N8" s="176"/>
-    </row>
-    <row r="9">
-      <c r="C9" s="172"/>
-      <c r="D9" s="172"/>
-      <c r="E9" s="172"/>
-      <c r="L9" s="176"/>
-      <c r="M9" s="176"/>
-      <c r="N9" s="176"/>
+      <c r="C8" s="220"/>
+      <c r="D8" s="220"/>
+      <c r="E8" s="220"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1535,7 +1457,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -1544,22 +1466,22 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>loss or report date changed</t>
+          <t>paid decreased</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="182"/>
-      <c r="D1" s="182"/>
-      <c r="E1" s="182"/>
+      <c r="C1" s="226"/>
+      <c r="D1" s="226"/>
+      <c r="E1" s="226"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
-      <c r="L1" s="186"/>
-      <c r="M1" s="186"/>
-      <c r="N1" s="186"/>
+      <c r="L1" s="230"/>
+      <c r="M1" s="230"/>
+      <c r="N1" s="230"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
@@ -1570,215 +1492,293 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be error correction, reopen, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="183"/>
-      <c r="D2" s="183"/>
-      <c r="E2" s="183"/>
-      <c r="L2" s="187"/>
-      <c r="M2" s="187"/>
-      <c r="N2" s="187"/>
+          <t>could be recoveries, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="227"/>
+      <c r="D2" s="227"/>
+      <c r="E2" s="227"/>
+      <c r="L2" s="231"/>
+      <c r="M2" s="231"/>
+      <c r="N2" s="231"/>
     </row>
     <row r="3">
-      <c r="C3" s="183"/>
-      <c r="D3" s="183"/>
-      <c r="E3" s="183"/>
-      <c r="L3" s="187"/>
-      <c r="M3" s="187"/>
-      <c r="N3" s="187"/>
+      <c r="C3" s="227"/>
+      <c r="D3" s="227"/>
+      <c r="E3" s="227"/>
+      <c r="L3" s="231"/>
+      <c r="M3" s="231"/>
+      <c r="N3" s="231"/>
     </row>
     <row r="4">
-      <c r="C4" s="183"/>
-      <c r="D4" s="183"/>
-      <c r="E4" s="183"/>
-      <c r="L4" s="187"/>
-      <c r="M4" s="187"/>
-      <c r="N4" s="187"/>
+      <c r="C4" s="227"/>
+      <c r="D4" s="227"/>
+      <c r="E4" s="227"/>
+      <c r="L4" s="231"/>
+      <c r="M4" s="231"/>
+      <c r="N4" s="231"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="181" t="inlineStr">
+      <c r="B5" s="225" t="inlineStr">
         <is>
           <t>claim_num.current</t>
         </is>
       </c>
-      <c r="C5" s="184" t="inlineStr">
+      <c r="C5" s="228" t="inlineStr">
         <is>
           <t>.currentc_date.c</t>
         </is>
       </c>
-      <c r="D5" s="184" t="inlineStr">
+      <c r="D5" s="228" t="inlineStr">
         <is>
           <t>r.prior_date.current</t>
         </is>
       </c>
-      <c r="E5" s="184" t="inlineStr">
+      <c r="E5" s="228" t="inlineStr">
         <is>
           <t>clsd_date.current</t>
         </is>
       </c>
-      <c r="F5" s="181" t="inlineStr">
+      <c r="F5" s="225" t="inlineStr">
         <is>
           <t>claim_status.current</t>
         </is>
       </c>
-      <c r="G5" s="181" t="inlineStr">
+      <c r="G5" s="225" t="inlineStr">
         <is>
           <t>r.prior_loss.current</t>
         </is>
       </c>
-      <c r="H5" s="181" t="inlineStr">
+      <c r="H5" s="225" t="inlineStr">
         <is>
           <t>pd_loss.current</t>
         </is>
       </c>
-      <c r="I5" s="181" t="inlineStr">
+      <c r="I5" s="225" t="inlineStr">
         <is>
           <t>case_loss.current</t>
         </is>
       </c>
-      <c r="J5" s="181" t="inlineStr">
+      <c r="J5" s="225" t="inlineStr">
         <is>
           <t>sou.currente.c</t>
         </is>
       </c>
-      <c r="K5" s="181" t="inlineStr">
+      <c r="K5" s="225" t="inlineStr">
         <is>
           <t>claim_num.prior</t>
         </is>
       </c>
-      <c r="L5" s="188" t="inlineStr">
+      <c r="L5" s="232" t="inlineStr">
         <is>
           <t>.currentc_date.prior</t>
         </is>
       </c>
-      <c r="M5" s="188" t="inlineStr">
+      <c r="M5" s="232" t="inlineStr">
         <is>
           <t>r.prior_date.p</t>
         </is>
       </c>
-      <c r="N5" s="188" t="inlineStr">
+      <c r="N5" s="232" t="inlineStr">
         <is>
           <t>clsd_date.prior</t>
         </is>
       </c>
-      <c r="O5" s="181" t="inlineStr">
+      <c r="O5" s="225" t="inlineStr">
         <is>
           <t>claim_status.prior</t>
         </is>
       </c>
-      <c r="P5" s="181" t="inlineStr">
+      <c r="P5" s="225" t="inlineStr">
         <is>
           <t>r.prior_loss.p</t>
         </is>
       </c>
-      <c r="Q5" s="181" t="inlineStr">
+      <c r="Q5" s="225" t="inlineStr">
         <is>
           <t>pd_loss.prior</t>
         </is>
       </c>
-      <c r="R5" s="181" t="inlineStr">
+      <c r="R5" s="225" t="inlineStr">
         <is>
           <t>case_loss.prior</t>
         </is>
       </c>
-      <c r="S5" s="181" t="inlineStr">
+      <c r="S5" s="225" t="inlineStr">
         <is>
           <t>sou.currente.prior</t>
         </is>
       </c>
-      <c r="T5" s="181"/>
+      <c r="T5" s="225"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B6" s="179" t="inlineStr">
-        <is>
-          <t>A0007</t>
-        </is>
-      </c>
-      <c r="C6" s="185">
-        <v>44064</v>
-      </c>
-      <c r="D6" s="185">
-        <v>44745</v>
-      </c>
-      <c r="E6" s="185">
-        <v>44757</v>
-      </c>
-      <c r="F6" s="179" t="inlineStr">
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="223" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C6" s="229">
+        <v>43499</v>
+      </c>
+      <c r="D6" s="229">
+        <v>43617</v>
+      </c>
+      <c r="E6" s="229">
+        <v>44217</v>
+      </c>
+      <c r="F6" s="223" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G6" s="179">
-        <v>7843</v>
-      </c>
-      <c r="H6" s="179">
-        <v>7843</v>
-      </c>
-      <c r="I6" s="179">
+      <c r="G6" s="223">
+        <v>72568</v>
+      </c>
+      <c r="H6" s="223">
+        <v>72568</v>
+      </c>
+      <c r="I6" s="223">
         <v>0</v>
       </c>
-      <c r="J6" s="179" t="inlineStr">
+      <c r="J6" s="223" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="179" t="inlineStr">
-        <is>
-          <t>A0007</t>
-        </is>
-      </c>
-      <c r="L6" s="189">
-        <v>44054</v>
-      </c>
-      <c r="M6" s="189">
-        <v>44745</v>
-      </c>
-      <c r="N6" s="189">
-        <v>44757</v>
-      </c>
-      <c r="O6" s="179" t="inlineStr">
+      <c r="K6" s="223" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="L6" s="233">
+        <v>43499</v>
+      </c>
+      <c r="M6" s="233">
+        <v>43617</v>
+      </c>
+      <c r="N6" s="233">
+        <v>44217</v>
+      </c>
+      <c r="O6" s="223" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="P6" s="179">
-        <v>7843</v>
-      </c>
-      <c r="Q6" s="179">
-        <v>7843</v>
-      </c>
-      <c r="R6" s="179">
+      <c r="P6" s="223">
+        <v>74570</v>
+      </c>
+      <c r="Q6" s="223">
+        <v>74570</v>
+      </c>
+      <c r="R6" s="223">
         <v>0</v>
       </c>
-      <c r="S6" s="179" t="inlineStr">
+      <c r="S6" s="223" t="inlineStr">
         <is>
           <t>ex1_prior</t>
         </is>
       </c>
-      <c r="T6" s="179"/>
+      <c r="T6" s="223"/>
     </row>
     <row r="7">
-      <c r="C7" s="183"/>
-      <c r="D7" s="183"/>
-      <c r="E7" s="183"/>
-      <c r="L7" s="187"/>
-      <c r="M7" s="187"/>
-      <c r="N7" s="187"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B7" s="223" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C7" s="229">
+        <v>44203</v>
+      </c>
+      <c r="D7" s="229">
+        <v>44245</v>
+      </c>
+      <c r="E7" s="229" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="223" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G7" s="223">
+        <v>78300</v>
+      </c>
+      <c r="H7" s="223">
+        <v>23792</v>
+      </c>
+      <c r="I7" s="223">
+        <v>54508</v>
+      </c>
+      <c r="J7" s="223" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="223" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="L7" s="233">
+        <v>44203</v>
+      </c>
+      <c r="M7" s="233">
+        <v>44245</v>
+      </c>
+      <c r="N7" s="233" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="223" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P7" s="223">
+        <v>78300</v>
+      </c>
+      <c r="Q7" s="223">
+        <v>25792</v>
+      </c>
+      <c r="R7" s="223">
+        <v>52508</v>
+      </c>
+      <c r="S7" s="223" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T7" s="223"/>
     </row>
     <row r="8">
-      <c r="C8" s="183"/>
-      <c r="D8" s="183"/>
-      <c r="E8" s="183"/>
-      <c r="L8" s="187"/>
-      <c r="M8" s="187"/>
-      <c r="N8" s="187"/>
+      <c r="C8" s="227"/>
+      <c r="D8" s="227"/>
+      <c r="E8" s="227"/>
+      <c r="L8" s="231"/>
+      <c r="M8" s="231"/>
+      <c r="N8" s="231"/>
+    </row>
+    <row r="9">
+      <c r="C9" s="227"/>
+      <c r="D9" s="227"/>
+      <c r="E9" s="227"/>
+      <c r="L9" s="231"/>
+      <c r="M9" s="231"/>
+      <c r="N9" s="231"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1801,22 +1801,22 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>claim number disappeared</t>
+          <t>loss or report date changed</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="193"/>
-      <c r="D1" s="193"/>
-      <c r="E1" s="193"/>
+      <c r="C1" s="237"/>
+      <c r="D1" s="237"/>
+      <c r="E1" s="237"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
-      <c r="L1" s="197"/>
-      <c r="M1" s="197"/>
-      <c r="N1" s="197"/>
+      <c r="L1" s="241"/>
+      <c r="M1" s="241"/>
+      <c r="N1" s="241"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
@@ -1827,229 +1827,215 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, rolling time window, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="L2" s="198"/>
-      <c r="M2" s="198"/>
-      <c r="N2" s="198"/>
+          <t>could be error correction, reopen, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="238"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="L2" s="242"/>
+      <c r="M2" s="242"/>
+      <c r="N2" s="242"/>
     </row>
     <row r="3">
-      <c r="C3" s="194"/>
-      <c r="D3" s="194"/>
-      <c r="E3" s="194"/>
-      <c r="L3" s="198"/>
-      <c r="M3" s="198"/>
-      <c r="N3" s="198"/>
+      <c r="C3" s="238"/>
+      <c r="D3" s="238"/>
+      <c r="E3" s="238"/>
+      <c r="L3" s="242"/>
+      <c r="M3" s="242"/>
+      <c r="N3" s="242"/>
     </row>
     <row r="4">
-      <c r="C4" s="194"/>
-      <c r="D4" s="194"/>
-      <c r="E4" s="194"/>
-      <c r="L4" s="198"/>
-      <c r="M4" s="198"/>
-      <c r="N4" s="198"/>
+      <c r="C4" s="238"/>
+      <c r="D4" s="238"/>
+      <c r="E4" s="238"/>
+      <c r="L4" s="242"/>
+      <c r="M4" s="242"/>
+      <c r="N4" s="242"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="192" t="inlineStr">
+      <c r="B5" s="236" t="inlineStr">
         <is>
           <t>claim_num.current</t>
         </is>
       </c>
-      <c r="C5" s="195" t="inlineStr">
+      <c r="C5" s="239" t="inlineStr">
         <is>
           <t>.currentc_date.c</t>
         </is>
       </c>
-      <c r="D5" s="195" t="inlineStr">
+      <c r="D5" s="239" t="inlineStr">
         <is>
           <t>r.prior_date.current</t>
         </is>
       </c>
-      <c r="E5" s="195" t="inlineStr">
+      <c r="E5" s="239" t="inlineStr">
         <is>
           <t>clsd_date.current</t>
         </is>
       </c>
-      <c r="F5" s="192" t="inlineStr">
+      <c r="F5" s="236" t="inlineStr">
         <is>
           <t>claim_status.current</t>
         </is>
       </c>
-      <c r="G5" s="192" t="inlineStr">
+      <c r="G5" s="236" t="inlineStr">
         <is>
           <t>r.prior_loss.current</t>
         </is>
       </c>
-      <c r="H5" s="192" t="inlineStr">
+      <c r="H5" s="236" t="inlineStr">
         <is>
           <t>pd_loss.current</t>
         </is>
       </c>
-      <c r="I5" s="192" t="inlineStr">
+      <c r="I5" s="236" t="inlineStr">
         <is>
           <t>case_loss.current</t>
         </is>
       </c>
-      <c r="J5" s="192" t="inlineStr">
+      <c r="J5" s="236" t="inlineStr">
         <is>
           <t>sou.currente.c</t>
         </is>
       </c>
-      <c r="K5" s="192" t="inlineStr">
+      <c r="K5" s="236" t="inlineStr">
         <is>
           <t>claim_num.prior</t>
         </is>
       </c>
-      <c r="L5" s="199" t="inlineStr">
+      <c r="L5" s="243" t="inlineStr">
         <is>
           <t>.currentc_date.prior</t>
         </is>
       </c>
-      <c r="M5" s="199" t="inlineStr">
+      <c r="M5" s="243" t="inlineStr">
         <is>
           <t>r.prior_date.p</t>
         </is>
       </c>
-      <c r="N5" s="199" t="inlineStr">
+      <c r="N5" s="243" t="inlineStr">
         <is>
           <t>clsd_date.prior</t>
         </is>
       </c>
-      <c r="O5" s="192" t="inlineStr">
+      <c r="O5" s="236" t="inlineStr">
         <is>
           <t>claim_status.prior</t>
         </is>
       </c>
-      <c r="P5" s="192" t="inlineStr">
+      <c r="P5" s="236" t="inlineStr">
         <is>
           <t>r.prior_loss.p</t>
         </is>
       </c>
-      <c r="Q5" s="192" t="inlineStr">
+      <c r="Q5" s="236" t="inlineStr">
         <is>
           <t>pd_loss.prior</t>
         </is>
       </c>
-      <c r="R5" s="192" t="inlineStr">
+      <c r="R5" s="236" t="inlineStr">
         <is>
           <t>case_loss.prior</t>
         </is>
       </c>
-      <c r="S5" s="192" t="inlineStr">
+      <c r="S5" s="236" t="inlineStr">
         <is>
           <t>sou.currente.prior</t>
         </is>
       </c>
-      <c r="T5" s="192"/>
+      <c r="T5" s="236"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C6" s="196" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D6" s="196" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E6" s="196" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J6" s="190" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K6" s="190" t="inlineStr">
-        <is>
-          <t>A0010</t>
-        </is>
-      </c>
-      <c r="L6" s="200">
-        <v>44312</v>
-      </c>
-      <c r="M6" s="200">
-        <v>44545</v>
-      </c>
-      <c r="N6" s="200" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O6" s="190" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="P6" s="190">
-        <v>17378</v>
-      </c>
-      <c r="Q6" s="190">
-        <v>12512</v>
-      </c>
-      <c r="R6" s="190">
-        <v>4866</v>
-      </c>
-      <c r="S6" s="190" t="inlineStr">
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" s="234" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="C6" s="240">
+        <v>44064</v>
+      </c>
+      <c r="D6" s="240">
+        <v>44745</v>
+      </c>
+      <c r="E6" s="240">
+        <v>44757</v>
+      </c>
+      <c r="F6" s="234" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="234">
+        <v>7843</v>
+      </c>
+      <c r="H6" s="234">
+        <v>7843</v>
+      </c>
+      <c r="I6" s="234">
+        <v>0</v>
+      </c>
+      <c r="J6" s="234" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="234" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="L6" s="244">
+        <v>44054</v>
+      </c>
+      <c r="M6" s="244">
+        <v>44745</v>
+      </c>
+      <c r="N6" s="244">
+        <v>44757</v>
+      </c>
+      <c r="O6" s="234" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P6" s="234">
+        <v>7843</v>
+      </c>
+      <c r="Q6" s="234">
+        <v>7843</v>
+      </c>
+      <c r="R6" s="234">
+        <v>0</v>
+      </c>
+      <c r="S6" s="234" t="inlineStr">
         <is>
           <t>ex1_prior</t>
         </is>
       </c>
-      <c r="T6" s="190"/>
+      <c r="T6" s="234"/>
     </row>
     <row r="7">
-      <c r="C7" s="194"/>
-      <c r="D7" s="194"/>
-      <c r="E7" s="194"/>
-      <c r="L7" s="198"/>
-      <c r="M7" s="198"/>
-      <c r="N7" s="198"/>
+      <c r="C7" s="238"/>
+      <c r="D7" s="238"/>
+      <c r="E7" s="238"/>
+      <c r="L7" s="242"/>
+      <c r="M7" s="242"/>
+      <c r="N7" s="242"/>
     </row>
     <row r="8">
-      <c r="C8" s="194"/>
-      <c r="D8" s="194"/>
-      <c r="E8" s="194"/>
-      <c r="L8" s="198"/>
-      <c r="M8" s="198"/>
-      <c r="N8" s="198"/>
+      <c r="C8" s="238"/>
+      <c r="D8" s="238"/>
+      <c r="E8" s="238"/>
+      <c r="L8" s="242"/>
+      <c r="M8" s="242"/>
+      <c r="N8" s="242"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -2063,321 +2049,264 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>error summary</t>
+          <t>claim number disappeared</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="C1" s="248"/>
+      <c r="D1" s="248"/>
+      <c r="E1" s="248"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="252"/>
+      <c r="M1" s="252"/>
+      <c r="N1" s="252"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>table of error types and counts</t>
-        </is>
-      </c>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, rolling time window, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="L2" s="253"/>
+      <c r="M2" s="253"/>
+      <c r="N2" s="253"/>
+    </row>
+    <row r="3">
+      <c r="C3" s="249"/>
+      <c r="D3" s="249"/>
+      <c r="E3" s="249"/>
+      <c r="L3" s="253"/>
+      <c r="M3" s="253"/>
+      <c r="N3" s="253"/>
+    </row>
+    <row r="4">
+      <c r="C4" s="249"/>
+      <c r="D4" s="249"/>
+      <c r="E4" s="249"/>
+      <c r="L4" s="253"/>
+      <c r="M4" s="253"/>
+      <c r="N4" s="253"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="202" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="202" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-      <c r="D5" s="202" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E5" s="202"/>
+      <c r="B5" s="247" t="inlineStr">
+        <is>
+          <t>claim_num.current</t>
+        </is>
+      </c>
+      <c r="C5" s="250" t="inlineStr">
+        <is>
+          <t>.currentc_date.c</t>
+        </is>
+      </c>
+      <c r="D5" s="250" t="inlineStr">
+        <is>
+          <t>r.prior_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="250" t="inlineStr">
+        <is>
+          <t>clsd_date.current</t>
+        </is>
+      </c>
+      <c r="F5" s="247" t="inlineStr">
+        <is>
+          <t>claim_status.current</t>
+        </is>
+      </c>
+      <c r="G5" s="247" t="inlineStr">
+        <is>
+          <t>r.prior_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="247" t="inlineStr">
+        <is>
+          <t>pd_loss.current</t>
+        </is>
+      </c>
+      <c r="I5" s="247" t="inlineStr">
+        <is>
+          <t>case_loss.current</t>
+        </is>
+      </c>
+      <c r="J5" s="247" t="inlineStr">
+        <is>
+          <t>sou.currente.c</t>
+        </is>
+      </c>
+      <c r="K5" s="247" t="inlineStr">
+        <is>
+          <t>claim_num.prior</t>
+        </is>
+      </c>
+      <c r="L5" s="254" t="inlineStr">
+        <is>
+          <t>.currentc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="254" t="inlineStr">
+        <is>
+          <t>r.prior_date.p</t>
+        </is>
+      </c>
+      <c r="N5" s="254" t="inlineStr">
+        <is>
+          <t>clsd_date.prior</t>
+        </is>
+      </c>
+      <c r="O5" s="247" t="inlineStr">
+        <is>
+          <t>claim_status.prior</t>
+        </is>
+      </c>
+      <c r="P5" s="247" t="inlineStr">
+        <is>
+          <t>r.prior_loss.p</t>
+        </is>
+      </c>
+      <c r="Q5" s="247" t="inlineStr">
+        <is>
+          <t>pd_loss.prior</t>
+        </is>
+      </c>
+      <c r="R5" s="247" t="inlineStr">
+        <is>
+          <t>case_loss.prior</t>
+        </is>
+      </c>
+      <c r="S5" s="247" t="inlineStr">
+        <is>
+          <t>sou.currente.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="247"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="201" t="inlineStr">
-        <is>
-          <t>claim numbers</t>
-        </is>
-      </c>
-      <c r="C6" s="201" t="inlineStr">
-        <is>
-          <t>claim numbers which potentially should show up but don't</t>
-        </is>
-      </c>
-      <c r="D6" s="201">
-        <v>1</v>
-      </c>
-      <c r="E6" s="201"/>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6" s="251" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D6" s="251" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E6" s="251" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" s="245" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K6" s="245" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="L6" s="255">
+        <v>44312</v>
+      </c>
+      <c r="M6" s="255">
+        <v>44545</v>
+      </c>
+      <c r="N6" s="255" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="245" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P6" s="245">
+        <v>17378</v>
+      </c>
+      <c r="Q6" s="245">
+        <v>12512</v>
+      </c>
+      <c r="R6" s="245">
+        <v>4866</v>
+      </c>
+      <c r="S6" s="245" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="245"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B7" s="201" t="inlineStr">
-        <is>
-          <t>claim dupes</t>
-        </is>
-      </c>
-      <c r="C7" s="201" t="inlineStr">
-        <is>
-          <t>claim numbers which show up multiple times</t>
-        </is>
-      </c>
-      <c r="D7" s="201">
-        <v>0</v>
-      </c>
-      <c r="E7" s="201"/>
+      <c r="C7" s="249"/>
+      <c r="D7" s="249"/>
+      <c r="E7" s="249"/>
+      <c r="L7" s="253"/>
+      <c r="M7" s="253"/>
+      <c r="N7" s="253"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="201" t="inlineStr">
-        <is>
-          <t>closure flag vs case</t>
-        </is>
-      </c>
-      <c r="C8" s="201" t="inlineStr">
-        <is>
-          <t>closure flag which doesn't seem to match case reserves</t>
-        </is>
-      </c>
-      <c r="D8" s="201">
-        <v>1</v>
-      </c>
-      <c r="E8" s="201"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B9" s="201" t="inlineStr">
-        <is>
-          <t>closure flag vs close date</t>
-        </is>
-      </c>
-      <c r="C9" s="201" t="inlineStr">
-        <is>
-          <t>closure flag which doesn't seem to match close date</t>
-        </is>
-      </c>
-      <c r="D9" s="201">
-        <v>0</v>
-      </c>
-      <c r="E9" s="201"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B10" s="201" t="inlineStr">
-        <is>
-          <t>close date &lt; report date</t>
-        </is>
-      </c>
-      <c r="C10" s="201" t="inlineStr">
-        <is>
-          <t>close date &lt; report date</t>
-        </is>
-      </c>
-      <c r="D10" s="201">
-        <v>0</v>
-      </c>
-      <c r="E10" s="201"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B11" s="201" t="inlineStr">
-        <is>
-          <t>report date &lt; loss date</t>
-        </is>
-      </c>
-      <c r="C11" s="201" t="inlineStr">
-        <is>
-          <t>report date &lt; loss date</t>
-        </is>
-      </c>
-      <c r="D11" s="201">
-        <v>0</v>
-      </c>
-      <c r="E11" s="201"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B12" s="201" t="inlineStr">
-        <is>
-          <t>missing loss or report date</t>
-        </is>
-      </c>
-      <c r="C12" s="201" t="inlineStr">
-        <is>
-          <t>missing loss or report date</t>
-        </is>
-      </c>
-      <c r="D12" s="201">
-        <v>0</v>
-      </c>
-      <c r="E12" s="201"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B13" s="201" t="inlineStr">
-        <is>
-          <t>negative paid or case</t>
-        </is>
-      </c>
-      <c r="C13" s="201" t="inlineStr">
-        <is>
-          <t>negative paid or case</t>
-        </is>
-      </c>
-      <c r="D13" s="201">
-        <v>0</v>
-      </c>
-      <c r="E13" s="201"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B14" s="201" t="inlineStr">
-        <is>
-          <t>paid+case vs rptd</t>
-        </is>
-      </c>
-      <c r="C14" s="201" t="inlineStr">
-        <is>
-          <t>paid+case vs rptd</t>
-        </is>
-      </c>
-      <c r="D14" s="201">
-        <v>1</v>
-      </c>
-      <c r="E14" s="201"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B15" s="201" t="inlineStr">
-        <is>
-          <t>paid decreased</t>
-        </is>
-      </c>
-      <c r="C15" s="201" t="inlineStr">
-        <is>
-          <t>paid decreased</t>
-        </is>
-      </c>
-      <c r="D15" s="201">
-        <v>2</v>
-      </c>
-      <c r="E15" s="201"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B16" s="201" t="inlineStr">
-        <is>
-          <t>loss or report date changed</t>
-        </is>
-      </c>
-      <c r="C16" s="201" t="inlineStr">
-        <is>
-          <t>loss or report date changed</t>
-        </is>
-      </c>
-      <c r="D16" s="201">
-        <v>1</v>
-      </c>
-      <c r="E16" s="201"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B17" s="201" t="inlineStr">
-        <is>
-          <t>claim number disappeared</t>
-        </is>
-      </c>
-      <c r="C17" s="201" t="inlineStr">
-        <is>
-          <t>claim number present in prior but not current</t>
-        </is>
-      </c>
-      <c r="D17" s="201">
-        <v>1</v>
-      </c>
-      <c r="E17" s="201"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B18" s="201" t="inlineStr">
-        <is>
-          <t>did we get new claims since last time?</t>
-        </is>
-      </c>
-      <c r="C18" s="201" t="inlineStr">
-        <is>
-          <t>1 if we got no new claims since prior loss run, else 0</t>
-        </is>
-      </c>
-      <c r="D18" s="201">
-        <v>0</v>
-      </c>
-      <c r="E18" s="201"/>
+      <c r="C8" s="249"/>
+      <c r="D8" s="249"/>
+      <c r="E8" s="249"/>
+      <c r="L8" s="253"/>
+      <c r="M8" s="253"/>
+      <c r="N8" s="253"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -4997,7 +4926,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -5006,77 +4935,312 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>claim numbers</t>
+          <t>error summary</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="150"/>
-      <c r="D1" s="150"/>
-      <c r="E1" s="151"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="151"/>
-      <c r="D2" s="151"/>
-      <c r="E2" s="151"/>
-    </row>
-    <row r="3">
-      <c r="C3" s="151"/>
-      <c r="D3" s="151"/>
-      <c r="E3" s="151"/>
-    </row>
-    <row r="4">
-      <c r="C4" s="151"/>
-      <c r="D4" s="151"/>
-      <c r="E4" s="151"/>
+          <t>table of error types and counts</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="149" t="inlineStr">
-        <is>
-          <t>claim_num.x</t>
-        </is>
-      </c>
-      <c r="C5" s="152" t="inlineStr">
-        <is>
-          <t>source.x</t>
-        </is>
-      </c>
-      <c r="D5" s="152"/>
-      <c r="E5" s="151"/>
+      <c r="B5" s="202" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C5" s="202" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D5" s="202" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E5" s="202"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="201" t="inlineStr">
+        <is>
+          <t>claim numbers</t>
+        </is>
+      </c>
+      <c r="C6" s="201" t="inlineStr">
+        <is>
+          <t>claim numbers which potentially should show up but don't</t>
+        </is>
+      </c>
+      <c r="D6" s="201">
+        <v>1</v>
+      </c>
+      <c r="E6" s="201"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="201" t="inlineStr">
+        <is>
+          <t>claim dupes</t>
+        </is>
+      </c>
+      <c r="C7" s="201" t="inlineStr">
+        <is>
+          <t>claim numbers which show up multiple times</t>
+        </is>
+      </c>
+      <c r="D7" s="201">
+        <v>0</v>
+      </c>
+      <c r="E7" s="201"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="201" t="inlineStr">
+        <is>
+          <t>closure flag vs case</t>
+        </is>
+      </c>
+      <c r="C8" s="201" t="inlineStr">
+        <is>
+          <t>closure flag which doesn't seem to match case reserves</t>
+        </is>
+      </c>
+      <c r="D8" s="201">
+        <v>1</v>
+      </c>
+      <c r="E8" s="201"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="201" t="inlineStr">
+        <is>
+          <t>closure flag vs close date</t>
+        </is>
+      </c>
+      <c r="C9" s="201" t="inlineStr">
+        <is>
+          <t>closure flag which doesn't seem to match close date</t>
+        </is>
+      </c>
+      <c r="D9" s="201">
+        <v>0</v>
+      </c>
+      <c r="E9" s="201"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="201" t="inlineStr">
+        <is>
+          <t>close date &lt; report date</t>
+        </is>
+      </c>
+      <c r="C10" s="201" t="inlineStr">
+        <is>
+          <t>close date &lt; report date</t>
+        </is>
+      </c>
+      <c r="D10" s="201">
+        <v>0</v>
+      </c>
+      <c r="E10" s="201"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="201" t="inlineStr">
+        <is>
+          <t>report date &lt; loss date</t>
+        </is>
+      </c>
+      <c r="C11" s="201" t="inlineStr">
+        <is>
+          <t>report date &lt; loss date</t>
+        </is>
+      </c>
+      <c r="D11" s="201">
+        <v>0</v>
+      </c>
+      <c r="E11" s="201"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" s="201" t="inlineStr">
+        <is>
+          <t>missing loss or report date</t>
+        </is>
+      </c>
+      <c r="C12" s="201" t="inlineStr">
+        <is>
+          <t>missing loss or report date</t>
+        </is>
+      </c>
+      <c r="D12" s="201">
+        <v>0</v>
+      </c>
+      <c r="E12" s="201"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" s="201" t="inlineStr">
+        <is>
+          <t>negative paid or case</t>
+        </is>
+      </c>
+      <c r="C13" s="201" t="inlineStr">
+        <is>
+          <t>negative paid or case</t>
+        </is>
+      </c>
+      <c r="D13" s="201">
+        <v>0</v>
+      </c>
+      <c r="E13" s="201"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" s="201" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="C14" s="201" t="inlineStr">
+        <is>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="D14" s="201">
+        <v>1</v>
+      </c>
+      <c r="E14" s="201"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B6" s="148" t="inlineStr">
-        <is>
-          <t>A0010</t>
-        </is>
-      </c>
-      <c r="C6" s="153" t="inlineStr">
-        <is>
-          <t>ex1_curr</t>
-        </is>
-      </c>
-      <c r="D6" s="153"/>
-      <c r="E6" s="151"/>
-    </row>
-    <row r="7">
-      <c r="C7" s="151"/>
-      <c r="D7" s="151"/>
-      <c r="E7" s="151"/>
-    </row>
-    <row r="8">
-      <c r="C8" s="151"/>
-      <c r="D8" s="151"/>
-      <c r="E8" s="151"/>
+      <c r="B15" s="201" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="C15" s="201" t="inlineStr">
+        <is>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="D15" s="201">
+        <v>2</v>
+      </c>
+      <c r="E15" s="201"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" s="201" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="C16" s="201" t="inlineStr">
+        <is>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="D16" s="201">
+        <v>1</v>
+      </c>
+      <c r="E16" s="201"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" s="201" t="inlineStr">
+        <is>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="C17" s="201" t="inlineStr">
+        <is>
+          <t>claim number present in prior but not current</t>
+        </is>
+      </c>
+      <c r="D17" s="201">
+        <v>1</v>
+      </c>
+      <c r="E17" s="201"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B18" s="201" t="inlineStr">
+        <is>
+          <t>did we get new claims since last time?</t>
+        </is>
+      </c>
+      <c r="C18" s="201" t="inlineStr">
+        <is>
+          <t>1 if we got no new claims since prior loss run, else 0</t>
+        </is>
+      </c>
+      <c r="D18" s="201">
+        <v>0</v>
+      </c>
+      <c r="E18" s="201"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -5090,103 +5254,57 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>closure flag vs case</t>
+          <t>claim numbers</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="206"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be something about claims process, timing issue, closure being defined at a different level of aggregation than the claim, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="206"/>
+      <c r="D2" s="206"/>
+      <c r="E2" s="206"/>
     </row>
     <row r="3">
-      <c r="C3" s="158"/>
-      <c r="D3" s="158"/>
-      <c r="E3" s="158"/>
+      <c r="C3" s="206"/>
+      <c r="D3" s="206"/>
+      <c r="E3" s="206"/>
     </row>
     <row r="4">
-      <c r="C4" s="158"/>
-      <c r="D4" s="158"/>
-      <c r="E4" s="158"/>
+      <c r="C4" s="206"/>
+      <c r="D4" s="206"/>
+      <c r="E4" s="206"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="156" t="inlineStr">
-        <is>
-          <t>claim_num</t>
-        </is>
-      </c>
-      <c r="C5" s="159" t="inlineStr">
-        <is>
-          <t>acc_date</t>
-        </is>
-      </c>
-      <c r="D5" s="159" t="inlineStr">
-        <is>
-          <t>rep_date</t>
-        </is>
-      </c>
-      <c r="E5" s="159" t="inlineStr">
-        <is>
-          <t>clsd_date</t>
-        </is>
-      </c>
-      <c r="F5" s="156" t="inlineStr">
-        <is>
-          <t>claim_status</t>
-        </is>
-      </c>
-      <c r="G5" s="156" t="inlineStr">
-        <is>
-          <t>rep_loss</t>
-        </is>
-      </c>
-      <c r="H5" s="156" t="inlineStr">
-        <is>
-          <t>pd_loss</t>
-        </is>
-      </c>
-      <c r="I5" s="156" t="inlineStr">
-        <is>
-          <t>case_loss</t>
-        </is>
-      </c>
-      <c r="J5" s="156" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K5" s="156" t="inlineStr">
-        <is>
-          <t>zero_case</t>
-        </is>
-      </c>
-      <c r="L5" s="156"/>
+      <c r="B5" s="204" t="inlineStr">
+        <is>
+          <t>claim_num.x</t>
+        </is>
+      </c>
+      <c r="C5" s="207" t="inlineStr">
+        <is>
+          <t>source.x</t>
+        </is>
+      </c>
+      <c r="D5" s="207"/>
+      <c r="E5" s="206"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -5194,53 +5312,28 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B6" s="154" t="inlineStr">
-        <is>
-          <t>A0011</t>
-        </is>
-      </c>
-      <c r="C6" s="160">
-        <v>44330</v>
-      </c>
-      <c r="D6" s="160">
-        <v>44853</v>
-      </c>
-      <c r="E6" s="160">
-        <v>44897</v>
-      </c>
-      <c r="F6" s="154" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="G6" s="154">
-        <v>62968</v>
-      </c>
-      <c r="H6" s="154">
-        <v>61968</v>
-      </c>
-      <c r="I6" s="154">
-        <v>1000</v>
-      </c>
-      <c r="J6" s="154" t="inlineStr">
+      <c r="B6" s="203" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="C6" s="208" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="154" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" s="154"/>
+      <c r="D6" s="208"/>
+      <c r="E6" s="206"/>
     </row>
     <row r="7">
-      <c r="C7" s="158"/>
-      <c r="D7" s="158"/>
-      <c r="E7" s="158"/>
+      <c r="C7" s="206"/>
+      <c r="D7" s="206"/>
+      <c r="E7" s="206"/>
     </row>
     <row r="8">
-      <c r="C8" s="158"/>
-      <c r="D8" s="158"/>
-      <c r="E8" s="158"/>
+      <c r="C8" s="206"/>
+      <c r="D8" s="206"/>
+      <c r="E8" s="206"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -5254,150 +5347,157 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="11" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>paid+case vs rptd</t>
+          <t>closure flag vs case</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="164"/>
-      <c r="D1" s="164"/>
-      <c r="E1" s="164"/>
+      <c r="C1" s="212"/>
+      <c r="D1" s="212"/>
+      <c r="E1" s="212"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be recoveries, expenses, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="165"/>
-      <c r="D2" s="165"/>
-      <c r="E2" s="165"/>
+          <t>could be something about claims process, timing issue, closure being defined at a different level of aggregation than the claim, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="213"/>
+      <c r="D2" s="213"/>
+      <c r="E2" s="213"/>
     </row>
     <row r="3">
-      <c r="C3" s="165"/>
-      <c r="D3" s="165"/>
-      <c r="E3" s="165"/>
+      <c r="C3" s="213"/>
+      <c r="D3" s="213"/>
+      <c r="E3" s="213"/>
     </row>
     <row r="4">
-      <c r="C4" s="165"/>
-      <c r="D4" s="165"/>
-      <c r="E4" s="165"/>
+      <c r="C4" s="213"/>
+      <c r="D4" s="213"/>
+      <c r="E4" s="213"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="163" t="inlineStr">
+      <c r="B5" s="211" t="inlineStr">
         <is>
           <t>claim_num</t>
         </is>
       </c>
-      <c r="C5" s="166" t="inlineStr">
+      <c r="C5" s="214" t="inlineStr">
         <is>
           <t>acc_date</t>
         </is>
       </c>
-      <c r="D5" s="166" t="inlineStr">
+      <c r="D5" s="214" t="inlineStr">
         <is>
           <t>rep_date</t>
         </is>
       </c>
-      <c r="E5" s="166" t="inlineStr">
+      <c r="E5" s="214" t="inlineStr">
         <is>
           <t>clsd_date</t>
         </is>
       </c>
-      <c r="F5" s="163" t="inlineStr">
+      <c r="F5" s="211" t="inlineStr">
         <is>
           <t>claim_status</t>
         </is>
       </c>
-      <c r="G5" s="163" t="inlineStr">
+      <c r="G5" s="211" t="inlineStr">
         <is>
           <t>rep_loss</t>
         </is>
       </c>
-      <c r="H5" s="163" t="inlineStr">
+      <c r="H5" s="211" t="inlineStr">
         <is>
           <t>pd_loss</t>
         </is>
       </c>
-      <c r="I5" s="163" t="inlineStr">
+      <c r="I5" s="211" t="inlineStr">
         <is>
           <t>case_loss</t>
         </is>
       </c>
-      <c r="J5" s="163" t="inlineStr">
+      <c r="J5" s="211" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="K5" s="163"/>
+      <c r="K5" s="211" t="inlineStr">
+        <is>
+          <t>zero_case</t>
+        </is>
+      </c>
+      <c r="L5" s="211"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" s="161" t="inlineStr">
-        <is>
-          <t>A0003</t>
-        </is>
-      </c>
-      <c r="C6" s="167">
-        <v>43704</v>
-      </c>
-      <c r="D6" s="167">
-        <v>44109</v>
-      </c>
-      <c r="E6" s="167" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" s="161" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G6" s="161">
-        <v>86564</v>
-      </c>
-      <c r="H6" s="161">
-        <v>78926</v>
-      </c>
-      <c r="I6" s="161">
-        <v>8638</v>
-      </c>
-      <c r="J6" s="161" t="inlineStr">
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" s="209" t="inlineStr">
+        <is>
+          <t>A0011</t>
+        </is>
+      </c>
+      <c r="C6" s="215">
+        <v>44330</v>
+      </c>
+      <c r="D6" s="215">
+        <v>44853</v>
+      </c>
+      <c r="E6" s="215">
+        <v>44897</v>
+      </c>
+      <c r="F6" s="209" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="209">
+        <v>62968</v>
+      </c>
+      <c r="H6" s="209">
+        <v>61968</v>
+      </c>
+      <c r="I6" s="209">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="209" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="161"/>
+      <c r="K6" s="209" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="209"/>
     </row>
     <row r="7">
-      <c r="C7" s="165"/>
-      <c r="D7" s="165"/>
-      <c r="E7" s="165"/>
+      <c r="C7" s="213"/>
+      <c r="D7" s="213"/>
+      <c r="E7" s="213"/>
     </row>
     <row r="8">
-      <c r="C8" s="165"/>
-      <c r="D8" s="165"/>
-      <c r="E8" s="165"/>
+      <c r="C8" s="213"/>
+      <c r="D8" s="213"/>
+      <c r="E8" s="213"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>

</xml_diff>

<commit_message>
fix naming in output
</commit_message>
<xml_diff>
--- a/output/PYRQ_output.xlsx
+++ b/output/PYRQ_output.xlsx
@@ -20,14 +20,14 @@
     <sheet name="triangles" sheetId="7" state="visible" r:id="rId5"/>
     <sheet name="notes" sheetId="8" state="visible" r:id="rId6"/>
     <sheet name="claim numbers" sheetId="9" state="visible" r:id="rId7"/>
-    <sheet name="retroactive changes" sheetId="15" state="visible" r:id="rId8"/>
-    <sheet name="maybe missing claims" sheetId="17" state="visible" r:id="rId9"/>
-    <sheet name="closure flag vs case" sheetId="18" state="visible" r:id="rId10"/>
-    <sheet name="paid+case vs rptd" sheetId="19" state="visible" r:id="rId11"/>
-    <sheet name="paid decreased" sheetId="20" state="visible" r:id="rId12"/>
-    <sheet name="loss or report date changed" sheetId="21" state="visible" r:id="rId13"/>
-    <sheet name="claim number disappeared" sheetId="22" state="visible" r:id="rId14"/>
-    <sheet name="error summary" sheetId="23" state="visible" r:id="rId15"/>
+    <sheet name="maybe missing claims" sheetId="51" state="visible" r:id="rId8"/>
+    <sheet name="closure flag vs case" sheetId="52" state="visible" r:id="rId9"/>
+    <sheet name="paid+case vs rptd" sheetId="53" state="visible" r:id="rId10"/>
+    <sheet name="paid decreased" sheetId="54" state="visible" r:id="rId11"/>
+    <sheet name="loss or report date changed" sheetId="55" state="visible" r:id="rId12"/>
+    <sheet name="claim number disappeared" sheetId="56" state="visible" r:id="rId13"/>
+    <sheet name="retroactive changes" sheetId="57" state="visible" r:id="rId14"/>
+    <sheet name="error summary" sheetId="58" state="visible" r:id="rId15"/>
   </sheets>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -130,7 +130,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="110">
+  <numFmts count="402">
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="###0"/>
     <numFmt numFmtId="168" formatCode="###0"/>
@@ -241,6 +241,298 @@
     <numFmt numFmtId="273" formatCode="YYYY\/MM\/DD"/>
     <numFmt numFmtId="274" formatCode="YYYY\/MM\/DD"/>
     <numFmt numFmtId="275" formatCode="#,##0"/>
+    <numFmt numFmtId="276" formatCode="#,##0"/>
+    <numFmt numFmtId="277" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="278" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="279" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="280" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="281" formatCode="#,##0"/>
+    <numFmt numFmtId="282" formatCode="#,##0"/>
+    <numFmt numFmtId="283" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="284" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="285" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="286" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="287" formatCode="#,##0"/>
+    <numFmt numFmtId="288" formatCode="#,##0"/>
+    <numFmt numFmtId="289" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="290" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="291" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="292" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="293" formatCode="#,##0"/>
+    <numFmt numFmtId="294" formatCode="#,##0"/>
+    <numFmt numFmtId="295" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="296" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="297" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="298" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="299" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="300" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="301" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="302" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="303" formatCode="#,##0"/>
+    <numFmt numFmtId="304" formatCode="#,##0"/>
+    <numFmt numFmtId="305" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="306" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="307" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="308" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="309" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="310" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="311" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="312" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="313" formatCode="#,##0"/>
+    <numFmt numFmtId="314" formatCode="#,##0"/>
+    <numFmt numFmtId="315" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="316" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="317" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="318" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="319" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="320" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="321" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="322" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="323" formatCode="#,##0"/>
+    <numFmt numFmtId="324" formatCode="#,##0"/>
+    <numFmt numFmtId="325" formatCode="#,##0"/>
+    <numFmt numFmtId="326" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="327" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="328" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="329" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="330" formatCode="#,##0"/>
+    <numFmt numFmtId="331" formatCode="#,##0"/>
+    <numFmt numFmtId="332" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="333" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="334" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="335" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="336" formatCode="#,##0"/>
+    <numFmt numFmtId="337" formatCode="#,##0"/>
+    <numFmt numFmtId="338" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="339" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="340" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="341" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="342" formatCode="#,##0"/>
+    <numFmt numFmtId="343" formatCode="#,##0"/>
+    <numFmt numFmtId="344" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="345" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="346" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="347" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="348" formatCode="#,##0"/>
+    <numFmt numFmtId="349" formatCode="#,##0"/>
+    <numFmt numFmtId="350" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="351" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="352" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="353" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="354" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="355" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="356" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="357" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="358" formatCode="#,##0"/>
+    <numFmt numFmtId="359" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="360" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="361" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="362" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="363" formatCode="#,##0"/>
+    <numFmt numFmtId="364" formatCode="#,##0"/>
+    <numFmt numFmtId="365" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="366" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="367" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="368" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="369" formatCode="#,##0"/>
+    <numFmt numFmtId="370" formatCode="#,##0"/>
+    <numFmt numFmtId="371" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="372" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="373" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="374" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="375" formatCode="#,##0"/>
+    <numFmt numFmtId="376" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="377" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="378" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="379" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="380" formatCode="#,##0"/>
+    <numFmt numFmtId="381" formatCode="#,##0"/>
+    <numFmt numFmtId="382" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="383" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="384" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="385" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="386" formatCode="#,##0"/>
+    <numFmt numFmtId="387" formatCode="#,##0"/>
+    <numFmt numFmtId="388" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="389" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="390" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="391" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="392" formatCode="#,##0"/>
+    <numFmt numFmtId="393" formatCode="#,##0"/>
+    <numFmt numFmtId="394" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="395" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="396" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="397" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="398" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="399" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="400" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="401" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="402" formatCode="#,##0"/>
+    <numFmt numFmtId="403" formatCode="#,##0"/>
+    <numFmt numFmtId="404" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="405" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="406" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="407" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="408" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="409" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="410" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="411" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="412" formatCode="#,##0"/>
+    <numFmt numFmtId="413" formatCode="#,##0"/>
+    <numFmt numFmtId="414" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="415" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="416" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="417" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="418" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="419" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="420" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="421" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="422" formatCode="#,##0"/>
+    <numFmt numFmtId="423" formatCode="#,##0"/>
+    <numFmt numFmtId="424" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="425" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="426" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="427" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="428" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="429" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="430" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="431" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="432" formatCode="#,##0"/>
+    <numFmt numFmtId="433" formatCode="#,##0"/>
+    <numFmt numFmtId="434" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="435" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="436" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="437" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="438" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="439" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="440" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="441" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="442" formatCode="#,##0"/>
+    <numFmt numFmtId="443" formatCode="#,##0"/>
+    <numFmt numFmtId="444" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="445" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="446" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="447" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="448" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="449" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="450" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="451" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="452" formatCode="#,##0"/>
+    <numFmt numFmtId="453" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="454" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="455" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="456" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="457" formatCode="#,##0"/>
+    <numFmt numFmtId="458" formatCode="#,##0"/>
+    <numFmt numFmtId="459" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="460" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="461" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="462" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="463" formatCode="#,##0"/>
+    <numFmt numFmtId="464" formatCode="#,##0"/>
+    <numFmt numFmtId="465" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="466" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="467" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="468" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="469" formatCode="#,##0"/>
+    <numFmt numFmtId="470" formatCode="#,##0"/>
+    <numFmt numFmtId="471" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="472" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="473" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="474" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="475" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="476" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="477" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="478" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="479" formatCode="#,##0"/>
+    <numFmt numFmtId="480" formatCode="#,##0"/>
+    <numFmt numFmtId="481" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="482" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="483" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="484" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="485" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="486" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="487" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="488" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="489" formatCode="#,##0"/>
+    <numFmt numFmtId="490" formatCode="#,##0"/>
+    <numFmt numFmtId="491" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="492" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="493" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="494" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="495" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="496" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="497" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="498" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="499" formatCode="#,##0"/>
+    <numFmt numFmtId="500" formatCode="#,##0"/>
+    <numFmt numFmtId="501" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="502" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="503" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="504" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="505" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="506" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="507" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="508" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="509" formatCode="#,##0"/>
+    <numFmt numFmtId="510" formatCode="#,##0"/>
+    <numFmt numFmtId="511" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="512" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="513" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="514" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="515" formatCode="#,##0"/>
+    <numFmt numFmtId="516" formatCode="#,##0"/>
+    <numFmt numFmtId="517" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="518" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="519" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="520" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="521" formatCode="#,##0"/>
+    <numFmt numFmtId="522" formatCode="#,##0"/>
+    <numFmt numFmtId="523" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="524" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="525" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="526" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="527" formatCode="#,##0"/>
+    <numFmt numFmtId="528" formatCode="#,##0"/>
+    <numFmt numFmtId="529" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="530" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="531" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="532" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="533" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="534" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="535" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="536" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="537" formatCode="#,##0"/>
+    <numFmt numFmtId="538" formatCode="#,##0"/>
+    <numFmt numFmtId="539" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="540" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="541" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="542" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="543" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="544" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="545" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="546" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="547" formatCode="#,##0"/>
+    <numFmt numFmtId="548" formatCode="#,##0"/>
+    <numFmt numFmtId="549" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="550" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="551" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="552" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="553" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="554" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="555" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="556" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="557" formatCode="#,##0"/>
+    <numFmt numFmtId="558" formatCode="#,##0"/>
+    <numFmt numFmtId="559" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="560" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="561" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="562" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="563" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="564" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="565" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="566" formatCode="YYYY\/MM\/DD"/>
+    <numFmt numFmtId="567" formatCode="#,##0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -263,12 +555,22 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF334E6F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8C8DC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -283,7 +585,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="589">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -416,6 +718,463 @@
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="274" xfId="0"/>
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="275" xfId="0"/>
     <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="275" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="276" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="276" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="277" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="278" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="279" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="280" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="281" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="282" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="281" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="283" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="284" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="285" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="286" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="287" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="288" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="287" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="289" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="290" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="291" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="292" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="293" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="294" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="293" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="295" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="296" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="297" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="298" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="299" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="300" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="301" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="302" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="303" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="304" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="303" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="305" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="306" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="307" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="308" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="309" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="310" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="311" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="312" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="313" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="314" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="313" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="315" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="316" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="317" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="318" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="319" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="320" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="321" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="322" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="323" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="323" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="324" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="325" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="324" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="326" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="327" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="328" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="329" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="330" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="331" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="330" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="332" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="333" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="334" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="335" xfId="0"/>
+    <xf applyFill="1" borderId="0" fillId="2" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="2" fontId="0" numFmtId="333" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="336" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="337" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="336" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="338" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="339" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="340" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="341" xfId="0"/>
+    <xf applyFill="1" borderId="0" fillId="3" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="339" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="342" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="343" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="342" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="344" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="345" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="346" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="347" xfId="0"/>
+    <xf applyFill="1" applyFont="1" borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="342" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="342" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="344" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="345" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="346" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="347" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="348" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="349" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="348" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="350" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="351" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="352" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="353" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="354" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="355" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="356" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="357" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="348" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="348" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="350" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="351" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="352" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="353" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="354" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="355" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="356" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="357" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="358" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="358" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="359" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="360" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="361" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="362" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="363" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="364" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="363" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="365" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="366" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="367" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="368" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="363" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="363" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="365" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="366" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="367" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="368" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="369" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="370" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="369" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="371" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="372" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="373" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="374" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="369" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="369" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="375" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="375" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="376" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="377" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="378" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="379" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="380" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="381" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="380" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="382" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="383" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="384" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="385" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="380" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="380" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="382" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="383" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="384" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="385" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="386" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="387" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="386" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="388" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="389" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="390" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="391" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="386" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="386" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="392" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="393" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="392" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="394" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="395" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="396" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="397" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="398" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="399" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="400" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="401" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="392" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="392" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="402" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="403" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="402" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="404" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="405" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="406" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="407" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="408" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="409" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="410" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="411" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="402" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="402" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="404" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="405" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="406" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="407" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="408" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="409" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="410" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="411" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="412" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="413" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="412" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="414" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="415" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="416" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="417" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="418" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="419" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="420" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="421" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="412" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="412" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="422" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="423" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="422" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="424" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="425" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="426" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="427" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="428" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="429" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="430" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="431" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="432" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="433" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="432" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="434" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="435" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="436" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="437" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="438" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="439" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="440" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="441" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="442" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="443" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="442" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="444" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="445" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="446" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="447" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="448" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="449" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="450" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="451" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="442" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="442" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="444" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="445" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="446" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="447" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="448" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="449" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="450" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="451" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="452" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="452" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="453" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="454" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="455" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="456" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="457" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="458" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="457" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="459" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="460" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="461" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="462" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="457" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="457" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="459" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="460" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="461" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="462" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="463" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="464" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="463" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="465" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="466" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="467" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="468" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="463" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="463" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="469" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="470" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="469" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="471" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="472" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="473" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="474" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="475" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="476" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="477" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="478" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="469" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="469" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="479" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="480" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="479" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="481" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="482" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="483" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="484" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="485" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="486" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="487" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="488" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="479" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="479" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="481" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="482" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="483" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="484" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="485" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="486" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="487" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="488" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="489" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="490" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="489" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="491" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="492" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="493" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="494" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="495" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="496" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="497" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="498" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="489" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="489" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="499" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="500" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="499" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="501" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="502" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="503" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="504" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="505" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="506" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="507" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="508" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="499" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="499" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="501" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="502" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="503" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="504" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="505" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="506" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="507" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="508" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="509" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="509" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="510" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="510" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="511" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="512" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="513" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="514" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="515" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="516" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="515" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="517" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="518" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="519" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="520" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="515" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="515" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="517" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="518" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="519" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="520" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="521" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="522" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="521" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="523" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="524" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="525" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="526" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="521" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="521" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="527" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="528" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="527" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="529" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="530" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="531" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="532" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="533" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="534" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="535" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="536" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="527" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="527" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="537" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="538" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="537" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="539" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="540" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="541" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="542" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="543" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="544" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="545" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="546" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="537" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="537" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="539" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="540" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="541" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="542" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="543" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="544" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="545" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="546" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="547" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="548" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="547" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="549" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="550" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="551" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="552" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="553" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="554" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="555" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="556" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="547" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="547" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="557" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="558" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="557" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="559" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="560" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="561" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="562" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="563" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="564" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="565" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="566" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="557" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="557" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="559" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="560" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="561" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="562" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="563" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="564" xfId="0"/>
+    <xf applyFill="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="2" numFmtId="565" xfId="0"/>
+    <xf applyFill="1" applyNumberFormat="1" borderId="0" fillId="3" fontId="0" numFmtId="566" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="567" xfId="0"/>
+    <xf applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="2" numFmtId="567" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1075,157 +1834,175 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="11" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>closure flag vs case</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
+          <t>paid+case vs rptd</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="513"/>
+      <c r="D1" s="513"/>
+      <c r="E1" s="513"/>
       <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
+      <c r="G1" s="219"/>
+      <c r="H1" s="219"/>
+      <c r="I1" s="219"/>
+      <c r="J1" s="219"/>
       <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be something about claims process, timing issue, closure being defined at a different level of aggregation than the claim, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
+          <t>could be recoveries, expenses, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="514"/>
+      <c r="D2" s="514"/>
+      <c r="E2" s="514"/>
+      <c r="G2" s="210"/>
+      <c r="H2" s="210"/>
+      <c r="I2" s="210"/>
+      <c r="J2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="514"/>
+      <c r="D3" s="514"/>
+      <c r="E3" s="514"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="87"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="514"/>
+      <c r="D4" s="514"/>
+      <c r="E4" s="514"/>
+      <c r="G4" s="210"/>
+      <c r="H4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="85" t="inlineStr">
+      <c r="B5" s="517" t="inlineStr">
         <is>
           <t>claim_num</t>
         </is>
       </c>
-      <c r="C5" s="88" t="inlineStr">
+      <c r="C5" s="515" t="inlineStr">
         <is>
           <t>acc_date</t>
         </is>
       </c>
-      <c r="D5" s="88" t="inlineStr">
+      <c r="D5" s="515" t="inlineStr">
         <is>
           <t>rep_date</t>
         </is>
       </c>
-      <c r="E5" s="88" t="inlineStr">
+      <c r="E5" s="515" t="inlineStr">
         <is>
           <t>clsd_date</t>
         </is>
       </c>
-      <c r="F5" s="85" t="inlineStr">
+      <c r="F5" s="512" t="inlineStr">
         <is>
           <t>claim_status</t>
         </is>
       </c>
-      <c r="G5" s="85" t="inlineStr">
+      <c r="G5" s="517" t="inlineStr">
         <is>
           <t>rep_loss</t>
         </is>
       </c>
-      <c r="H5" s="85" t="inlineStr">
+      <c r="H5" s="517" t="inlineStr">
         <is>
           <t>pd_loss</t>
         </is>
       </c>
-      <c r="I5" s="85" t="inlineStr">
+      <c r="I5" s="517" t="inlineStr">
         <is>
           <t>case_loss</t>
         </is>
       </c>
-      <c r="J5" s="85" t="inlineStr">
+      <c r="J5" s="517" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="K5" s="85" t="inlineStr">
-        <is>
-          <t>zero_case</t>
-        </is>
-      </c>
-      <c r="L5" s="85"/>
+      <c r="K5" s="512"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B6" s="83" t="inlineStr">
-        <is>
-          <t>A0011</t>
-        </is>
-      </c>
-      <c r="C6" s="89">
-        <v>44330</v>
-      </c>
-      <c r="D6" s="89">
-        <v>44853</v>
-      </c>
-      <c r="E6" s="89">
-        <v>44897</v>
-      </c>
-      <c r="F6" s="83" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="G6" s="83">
-        <v>62968</v>
-      </c>
-      <c r="H6" s="83">
-        <v>61968</v>
-      </c>
-      <c r="I6" s="83">
-        <v>1000</v>
-      </c>
-      <c r="J6" s="83" t="inlineStr">
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="518" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C6" s="516">
+        <v>43704</v>
+      </c>
+      <c r="D6" s="516">
+        <v>44109</v>
+      </c>
+      <c r="E6" s="516" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="510" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G6" s="518">
+        <v>86564</v>
+      </c>
+      <c r="H6" s="518">
+        <v>78926</v>
+      </c>
+      <c r="I6" s="518">
+        <v>8638</v>
+      </c>
+      <c r="J6" s="518" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="83" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" s="83"/>
+      <c r="K6" s="510"/>
     </row>
     <row r="7">
-      <c r="C7" s="87"/>
-      <c r="D7" s="87"/>
-      <c r="E7" s="87"/>
+      <c r="B7" s="210"/>
+      <c r="C7" s="514"/>
+      <c r="D7" s="514"/>
+      <c r="E7" s="514"/>
+      <c r="G7" s="210"/>
+      <c r="H7" s="210"/>
+      <c r="I7" s="210"/>
+      <c r="J7" s="210"/>
     </row>
     <row r="8">
-      <c r="C8" s="87"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="87"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="514"/>
+      <c r="D8" s="514"/>
+      <c r="E8" s="514"/>
+      <c r="G8" s="210"/>
+      <c r="H8" s="210"/>
+      <c r="I8" s="210"/>
+      <c r="J8" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1239,150 +2016,358 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="11" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>paid+case vs rptd</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
+          <t>paid decreased</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="522"/>
+      <c r="D1" s="522"/>
+      <c r="E1" s="522"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="H1" s="219"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="219"/>
+      <c r="L1" s="526"/>
+      <c r="M1" s="526"/>
+      <c r="N1" s="526"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="219"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="219"/>
+      <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be recoveries, expenses, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
+          <t>could be recoveries, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="523"/>
+      <c r="D2" s="523"/>
+      <c r="E2" s="523"/>
+      <c r="H2" s="210"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="527"/>
+      <c r="M2" s="527"/>
+      <c r="N2" s="527"/>
+      <c r="Q2" s="210"/>
+      <c r="S2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="523"/>
+      <c r="D3" s="523"/>
+      <c r="E3" s="523"/>
+      <c r="H3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="527"/>
+      <c r="M3" s="527"/>
+      <c r="N3" s="527"/>
+      <c r="Q3" s="210"/>
+      <c r="S3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="94"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="94"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="523"/>
+      <c r="D4" s="523"/>
+      <c r="E4" s="523"/>
+      <c r="H4" s="210"/>
+      <c r="J4" s="210"/>
+      <c r="K4" s="210"/>
+      <c r="L4" s="527"/>
+      <c r="M4" s="527"/>
+      <c r="N4" s="527"/>
+      <c r="Q4" s="210"/>
+      <c r="S4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="92" t="inlineStr">
-        <is>
-          <t>claim_num</t>
-        </is>
-      </c>
-      <c r="C5" s="95" t="inlineStr">
-        <is>
-          <t>acc_date</t>
-        </is>
-      </c>
-      <c r="D5" s="95" t="inlineStr">
-        <is>
-          <t>rep_date</t>
-        </is>
-      </c>
-      <c r="E5" s="95" t="inlineStr">
-        <is>
-          <t>clsd_date</t>
-        </is>
-      </c>
-      <c r="F5" s="92" t="inlineStr">
-        <is>
-          <t>claim_status</t>
-        </is>
-      </c>
-      <c r="G5" s="92" t="inlineStr">
-        <is>
-          <t>rep_loss</t>
-        </is>
-      </c>
-      <c r="H5" s="92" t="inlineStr">
-        <is>
-          <t>pd_loss</t>
-        </is>
-      </c>
-      <c r="I5" s="92" t="inlineStr">
-        <is>
-          <t>case_loss</t>
-        </is>
-      </c>
-      <c r="J5" s="92" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K5" s="92"/>
+      <c r="B5" s="530" t="inlineStr">
+        <is>
+          <t>claim_num.current</t>
+        </is>
+      </c>
+      <c r="C5" s="524" t="inlineStr">
+        <is>
+          <t>acc_date.current</t>
+        </is>
+      </c>
+      <c r="D5" s="524" t="inlineStr">
+        <is>
+          <t>rep_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="524" t="inlineStr">
+        <is>
+          <t>clsd_date.current</t>
+        </is>
+      </c>
+      <c r="F5" s="521" t="inlineStr">
+        <is>
+          <t>claim_status.current</t>
+        </is>
+      </c>
+      <c r="G5" s="521" t="inlineStr">
+        <is>
+          <t>rep_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="530" t="inlineStr">
+        <is>
+          <t>pd_loss.current</t>
+        </is>
+      </c>
+      <c r="I5" s="521" t="inlineStr">
+        <is>
+          <t>case_loss.current</t>
+        </is>
+      </c>
+      <c r="J5" s="530" t="inlineStr">
+        <is>
+          <t>source.current</t>
+        </is>
+      </c>
+      <c r="K5" s="530" t="inlineStr">
+        <is>
+          <t>claim_num.prior</t>
+        </is>
+      </c>
+      <c r="L5" s="528" t="inlineStr">
+        <is>
+          <t>acc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="528" t="inlineStr">
+        <is>
+          <t>rep_date.prior</t>
+        </is>
+      </c>
+      <c r="N5" s="528" t="inlineStr">
+        <is>
+          <t>clsd_date.prior</t>
+        </is>
+      </c>
+      <c r="O5" s="521" t="inlineStr">
+        <is>
+          <t>claim_status.prior</t>
+        </is>
+      </c>
+      <c r="P5" s="521" t="inlineStr">
+        <is>
+          <t>rep_loss.prior</t>
+        </is>
+      </c>
+      <c r="Q5" s="530" t="inlineStr">
+        <is>
+          <t>pd_loss.prior</t>
+        </is>
+      </c>
+      <c r="R5" s="521" t="inlineStr">
+        <is>
+          <t>case_loss.prior</t>
+        </is>
+      </c>
+      <c r="S5" s="530" t="inlineStr">
+        <is>
+          <t>source.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="521"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" s="90" t="inlineStr">
-        <is>
-          <t>A0003</t>
-        </is>
-      </c>
-      <c r="C6" s="96">
-        <v>43704</v>
-      </c>
-      <c r="D6" s="96">
-        <v>44109</v>
-      </c>
-      <c r="E6" s="96" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" s="90" t="inlineStr">
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="531" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C6" s="525">
+        <v>43499</v>
+      </c>
+      <c r="D6" s="525">
+        <v>43617</v>
+      </c>
+      <c r="E6" s="525">
+        <v>44217</v>
+      </c>
+      <c r="F6" s="519" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="519">
+        <v>72568</v>
+      </c>
+      <c r="H6" s="531">
+        <v>72568</v>
+      </c>
+      <c r="I6" s="519">
+        <v>0</v>
+      </c>
+      <c r="J6" s="531" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="531" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="L6" s="529">
+        <v>43499</v>
+      </c>
+      <c r="M6" s="529">
+        <v>43617</v>
+      </c>
+      <c r="N6" s="529">
+        <v>44217</v>
+      </c>
+      <c r="O6" s="519" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="P6" s="519">
+        <v>74570</v>
+      </c>
+      <c r="Q6" s="531">
+        <v>74570</v>
+      </c>
+      <c r="R6" s="519">
+        <v>0</v>
+      </c>
+      <c r="S6" s="531" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T6" s="519"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B7" s="531" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C7" s="525">
+        <v>44203</v>
+      </c>
+      <c r="D7" s="525">
+        <v>44245</v>
+      </c>
+      <c r="E7" s="525" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="519" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G6" s="90">
-        <v>86564</v>
-      </c>
-      <c r="H6" s="90">
-        <v>78926</v>
-      </c>
-      <c r="I6" s="90">
-        <v>8638</v>
-      </c>
-      <c r="J6" s="90" t="inlineStr">
+      <c r="G7" s="519">
+        <v>78300</v>
+      </c>
+      <c r="H7" s="531">
+        <v>23792</v>
+      </c>
+      <c r="I7" s="519">
+        <v>54508</v>
+      </c>
+      <c r="J7" s="531" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="90"/>
-    </row>
-    <row r="7">
-      <c r="C7" s="94"/>
-      <c r="D7" s="94"/>
-      <c r="E7" s="94"/>
+      <c r="K7" s="531" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="L7" s="529">
+        <v>44203</v>
+      </c>
+      <c r="M7" s="529">
+        <v>44245</v>
+      </c>
+      <c r="N7" s="529" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="519" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P7" s="519">
+        <v>78300</v>
+      </c>
+      <c r="Q7" s="531">
+        <v>25792</v>
+      </c>
+      <c r="R7" s="519">
+        <v>52508</v>
+      </c>
+      <c r="S7" s="531" t="inlineStr">
+        <is>
+          <t>ex1_prior</t>
+        </is>
+      </c>
+      <c r="T7" s="519"/>
     </row>
     <row r="8">
-      <c r="C8" s="94"/>
-      <c r="D8" s="94"/>
-      <c r="E8" s="94"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="523"/>
+      <c r="D8" s="523"/>
+      <c r="E8" s="523"/>
+      <c r="H8" s="210"/>
+      <c r="J8" s="210"/>
+      <c r="K8" s="210"/>
+      <c r="L8" s="527"/>
+      <c r="M8" s="527"/>
+      <c r="N8" s="527"/>
+      <c r="Q8" s="210"/>
+      <c r="S8" s="210"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="210"/>
+      <c r="C9" s="523"/>
+      <c r="D9" s="523"/>
+      <c r="E9" s="523"/>
+      <c r="H9" s="210"/>
+      <c r="J9" s="210"/>
+      <c r="K9" s="210"/>
+      <c r="L9" s="527"/>
+      <c r="M9" s="527"/>
+      <c r="N9" s="527"/>
+      <c r="Q9" s="210"/>
+      <c r="S9" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1396,7 +2381,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -1405,319 +2390,261 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>paid decreased</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
+          <t>loss or report date changed</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="545"/>
+      <c r="D1" s="545"/>
+      <c r="E1" s="535"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="104"/>
-      <c r="M1" s="104"/>
-      <c r="N1" s="104"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="219"/>
+      <c r="L1" s="549"/>
+      <c r="M1" s="549"/>
+      <c r="N1" s="539"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
+      <c r="S1" s="219"/>
       <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be recoveries, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
-      <c r="N2" s="105"/>
+          <t>could be error correction, reopen, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="546"/>
+      <c r="D2" s="546"/>
+      <c r="E2" s="536"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="550"/>
+      <c r="M2" s="550"/>
+      <c r="N2" s="540"/>
+      <c r="S2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
-      <c r="N3" s="105"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="546"/>
+      <c r="D3" s="546"/>
+      <c r="E3" s="536"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="550"/>
+      <c r="M3" s="550"/>
+      <c r="N3" s="540"/>
+      <c r="S3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="101"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="101"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="105"/>
-      <c r="N4" s="105"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="546"/>
+      <c r="D4" s="546"/>
+      <c r="E4" s="536"/>
+      <c r="J4" s="210"/>
+      <c r="K4" s="210"/>
+      <c r="L4" s="550"/>
+      <c r="M4" s="550"/>
+      <c r="N4" s="540"/>
+      <c r="S4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="99" t="inlineStr">
+      <c r="B5" s="543" t="inlineStr">
         <is>
           <t>claim_num.current</t>
         </is>
       </c>
-      <c r="C5" s="102" t="inlineStr">
-        <is>
-          <t>.currentc_date.c</t>
-        </is>
-      </c>
-      <c r="D5" s="102" t="inlineStr">
-        <is>
-          <t>r.prior_date.current</t>
-        </is>
-      </c>
-      <c r="E5" s="102" t="inlineStr">
+      <c r="C5" s="547" t="inlineStr">
+        <is>
+          <t>acc_date.current</t>
+        </is>
+      </c>
+      <c r="D5" s="547" t="inlineStr">
+        <is>
+          <t>rep_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="537" t="inlineStr">
         <is>
           <t>clsd_date.current</t>
         </is>
       </c>
-      <c r="F5" s="99" t="inlineStr">
+      <c r="F5" s="534" t="inlineStr">
         <is>
           <t>claim_status.current</t>
         </is>
       </c>
-      <c r="G5" s="99" t="inlineStr">
-        <is>
-          <t>r.prior_loss.current</t>
-        </is>
-      </c>
-      <c r="H5" s="99" t="inlineStr">
+      <c r="G5" s="534" t="inlineStr">
+        <is>
+          <t>rep_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="534" t="inlineStr">
         <is>
           <t>pd_loss.current</t>
         </is>
       </c>
-      <c r="I5" s="99" t="inlineStr">
+      <c r="I5" s="534" t="inlineStr">
         <is>
           <t>case_loss.current</t>
         </is>
       </c>
-      <c r="J5" s="99" t="inlineStr">
-        <is>
-          <t>sou.currente.c</t>
-        </is>
-      </c>
-      <c r="K5" s="99" t="inlineStr">
+      <c r="J5" s="543" t="inlineStr">
+        <is>
+          <t>source.current</t>
+        </is>
+      </c>
+      <c r="K5" s="543" t="inlineStr">
         <is>
           <t>claim_num.prior</t>
         </is>
       </c>
-      <c r="L5" s="106" t="inlineStr">
-        <is>
-          <t>.currentc_date.prior</t>
-        </is>
-      </c>
-      <c r="M5" s="106" t="inlineStr">
-        <is>
-          <t>r.prior_date.p</t>
-        </is>
-      </c>
-      <c r="N5" s="106" t="inlineStr">
+      <c r="L5" s="551" t="inlineStr">
+        <is>
+          <t>acc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="551" t="inlineStr">
+        <is>
+          <t>rep_date.prior</t>
+        </is>
+      </c>
+      <c r="N5" s="541" t="inlineStr">
         <is>
           <t>clsd_date.prior</t>
         </is>
       </c>
-      <c r="O5" s="99" t="inlineStr">
+      <c r="O5" s="534" t="inlineStr">
         <is>
           <t>claim_status.prior</t>
         </is>
       </c>
-      <c r="P5" s="99" t="inlineStr">
-        <is>
-          <t>r.prior_loss.p</t>
-        </is>
-      </c>
-      <c r="Q5" s="99" t="inlineStr">
+      <c r="P5" s="534" t="inlineStr">
+        <is>
+          <t>rep_loss.prior</t>
+        </is>
+      </c>
+      <c r="Q5" s="534" t="inlineStr">
         <is>
           <t>pd_loss.prior</t>
         </is>
       </c>
-      <c r="R5" s="99" t="inlineStr">
+      <c r="R5" s="534" t="inlineStr">
         <is>
           <t>case_loss.prior</t>
         </is>
       </c>
-      <c r="S5" s="99" t="inlineStr">
-        <is>
-          <t>sou.currente.prior</t>
-        </is>
-      </c>
-      <c r="T5" s="99"/>
+      <c r="S5" s="543" t="inlineStr">
+        <is>
+          <t>source.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="534"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="97" t="inlineStr">
-        <is>
-          <t>A0001</t>
-        </is>
-      </c>
-      <c r="C6" s="103">
-        <v>43499</v>
-      </c>
-      <c r="D6" s="103">
-        <v>43617</v>
-      </c>
-      <c r="E6" s="103">
-        <v>44217</v>
-      </c>
-      <c r="F6" s="97" t="inlineStr">
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" s="544" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="C6" s="548">
+        <v>44064</v>
+      </c>
+      <c r="D6" s="548">
+        <v>44745</v>
+      </c>
+      <c r="E6" s="538">
+        <v>44757</v>
+      </c>
+      <c r="F6" s="532" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G6" s="97">
-        <v>72568</v>
-      </c>
-      <c r="H6" s="97">
-        <v>72568</v>
-      </c>
-      <c r="I6" s="97">
+      <c r="G6" s="532">
+        <v>7843</v>
+      </c>
+      <c r="H6" s="532">
+        <v>7843</v>
+      </c>
+      <c r="I6" s="532">
         <v>0</v>
       </c>
-      <c r="J6" s="97" t="inlineStr">
+      <c r="J6" s="544" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="K6" s="97" t="inlineStr">
-        <is>
-          <t>A0001</t>
-        </is>
-      </c>
-      <c r="L6" s="107">
-        <v>43499</v>
-      </c>
-      <c r="M6" s="107">
-        <v>43617</v>
-      </c>
-      <c r="N6" s="107">
-        <v>44217</v>
-      </c>
-      <c r="O6" s="97" t="inlineStr">
+      <c r="K6" s="544" t="inlineStr">
+        <is>
+          <t>A0007</t>
+        </is>
+      </c>
+      <c r="L6" s="552">
+        <v>44054</v>
+      </c>
+      <c r="M6" s="552">
+        <v>44745</v>
+      </c>
+      <c r="N6" s="542">
+        <v>44757</v>
+      </c>
+      <c r="O6" s="532" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="P6" s="97">
-        <v>74570</v>
-      </c>
-      <c r="Q6" s="97">
-        <v>74570</v>
-      </c>
-      <c r="R6" s="97">
+      <c r="P6" s="532">
+        <v>7843</v>
+      </c>
+      <c r="Q6" s="532">
+        <v>7843</v>
+      </c>
+      <c r="R6" s="532">
         <v>0</v>
       </c>
-      <c r="S6" s="97" t="inlineStr">
+      <c r="S6" s="544" t="inlineStr">
         <is>
           <t>ex1_prior</t>
         </is>
       </c>
-      <c r="T6" s="97"/>
+      <c r="T6" s="532"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B7" s="97" t="inlineStr">
-        <is>
-          <t>A0008</t>
-        </is>
-      </c>
-      <c r="C7" s="103">
-        <v>44203</v>
-      </c>
-      <c r="D7" s="103">
-        <v>44245</v>
-      </c>
-      <c r="E7" s="103" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" s="97" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G7" s="97">
-        <v>78300</v>
-      </c>
-      <c r="H7" s="97">
-        <v>23792</v>
-      </c>
-      <c r="I7" s="97">
-        <v>54508</v>
-      </c>
-      <c r="J7" s="97" t="inlineStr">
-        <is>
-          <t>ex1_curr</t>
-        </is>
-      </c>
-      <c r="K7" s="97" t="inlineStr">
-        <is>
-          <t>A0008</t>
-        </is>
-      </c>
-      <c r="L7" s="107">
-        <v>44203</v>
-      </c>
-      <c r="M7" s="107">
-        <v>44245</v>
-      </c>
-      <c r="N7" s="107" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O7" s="97" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="P7" s="97">
-        <v>78300</v>
-      </c>
-      <c r="Q7" s="97">
-        <v>25792</v>
-      </c>
-      <c r="R7" s="97">
-        <v>52508</v>
-      </c>
-      <c r="S7" s="97" t="inlineStr">
-        <is>
-          <t>ex1_prior</t>
-        </is>
-      </c>
-      <c r="T7" s="97"/>
+      <c r="B7" s="210"/>
+      <c r="C7" s="546"/>
+      <c r="D7" s="546"/>
+      <c r="E7" s="536"/>
+      <c r="J7" s="210"/>
+      <c r="K7" s="210"/>
+      <c r="L7" s="550"/>
+      <c r="M7" s="550"/>
+      <c r="N7" s="540"/>
+      <c r="S7" s="210"/>
     </row>
     <row r="8">
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="L8" s="105"/>
-      <c r="M8" s="105"/>
-      <c r="N8" s="105"/>
-    </row>
-    <row r="9">
-      <c r="C9" s="101"/>
-      <c r="D9" s="101"/>
-      <c r="E9" s="101"/>
-      <c r="L9" s="105"/>
-      <c r="M9" s="105"/>
-      <c r="N9" s="105"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="546"/>
+      <c r="D8" s="546"/>
+      <c r="E8" s="536"/>
+      <c r="J8" s="210"/>
+      <c r="K8" s="210"/>
+      <c r="L8" s="550"/>
+      <c r="M8" s="550"/>
+      <c r="N8" s="540"/>
+      <c r="S8" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1740,241 +2667,275 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>loss or report date changed</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
+          <t>claim number disappeared</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="556"/>
+      <c r="D1" s="556"/>
+      <c r="E1" s="556"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="115"/>
-      <c r="M1" s="115"/>
-      <c r="N1" s="115"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="219"/>
+      <c r="L1" s="560"/>
+      <c r="M1" s="560"/>
+      <c r="N1" s="560"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
+      <c r="S1" s="219"/>
       <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be error correction, reopen, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, rolling time window, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="557"/>
+      <c r="D2" s="557"/>
+      <c r="E2" s="557"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="561"/>
+      <c r="M2" s="561"/>
+      <c r="N2" s="561"/>
+      <c r="S2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="112"/>
-      <c r="D3" s="112"/>
-      <c r="E3" s="112"/>
-      <c r="L3" s="116"/>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="557"/>
+      <c r="D3" s="557"/>
+      <c r="E3" s="557"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="561"/>
+      <c r="M3" s="561"/>
+      <c r="N3" s="561"/>
+      <c r="S3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="112"/>
-      <c r="D4" s="112"/>
-      <c r="E4" s="112"/>
-      <c r="L4" s="116"/>
-      <c r="M4" s="116"/>
-      <c r="N4" s="116"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="557"/>
+      <c r="D4" s="557"/>
+      <c r="E4" s="557"/>
+      <c r="J4" s="210"/>
+      <c r="K4" s="210"/>
+      <c r="L4" s="561"/>
+      <c r="M4" s="561"/>
+      <c r="N4" s="561"/>
+      <c r="S4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="110" t="inlineStr">
+      <c r="B5" s="564" t="inlineStr">
         <is>
           <t>claim_num.current</t>
         </is>
       </c>
-      <c r="C5" s="113" t="inlineStr">
-        <is>
-          <t>.currentc_date.c</t>
-        </is>
-      </c>
-      <c r="D5" s="113" t="inlineStr">
-        <is>
-          <t>r.prior_date.current</t>
-        </is>
-      </c>
-      <c r="E5" s="113" t="inlineStr">
+      <c r="C5" s="558" t="inlineStr">
+        <is>
+          <t>acc_date.current</t>
+        </is>
+      </c>
+      <c r="D5" s="558" t="inlineStr">
+        <is>
+          <t>rep_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="558" t="inlineStr">
         <is>
           <t>clsd_date.current</t>
         </is>
       </c>
-      <c r="F5" s="110" t="inlineStr">
+      <c r="F5" s="555" t="inlineStr">
         <is>
           <t>claim_status.current</t>
         </is>
       </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>r.prior_loss.current</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
+      <c r="G5" s="555" t="inlineStr">
+        <is>
+          <t>rep_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="555" t="inlineStr">
         <is>
           <t>pd_loss.current</t>
         </is>
       </c>
-      <c r="I5" s="110" t="inlineStr">
+      <c r="I5" s="555" t="inlineStr">
         <is>
           <t>case_loss.current</t>
         </is>
       </c>
-      <c r="J5" s="110" t="inlineStr">
-        <is>
-          <t>sou.currente.c</t>
-        </is>
-      </c>
-      <c r="K5" s="110" t="inlineStr">
+      <c r="J5" s="564" t="inlineStr">
+        <is>
+          <t>source.current</t>
+        </is>
+      </c>
+      <c r="K5" s="564" t="inlineStr">
         <is>
           <t>claim_num.prior</t>
         </is>
       </c>
-      <c r="L5" s="117" t="inlineStr">
-        <is>
-          <t>.currentc_date.prior</t>
-        </is>
-      </c>
-      <c r="M5" s="117" t="inlineStr">
-        <is>
-          <t>r.prior_date.p</t>
-        </is>
-      </c>
-      <c r="N5" s="117" t="inlineStr">
+      <c r="L5" s="562" t="inlineStr">
+        <is>
+          <t>acc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="562" t="inlineStr">
+        <is>
+          <t>rep_date.prior</t>
+        </is>
+      </c>
+      <c r="N5" s="562" t="inlineStr">
         <is>
           <t>clsd_date.prior</t>
         </is>
       </c>
-      <c r="O5" s="110" t="inlineStr">
+      <c r="O5" s="555" t="inlineStr">
         <is>
           <t>claim_status.prior</t>
         </is>
       </c>
-      <c r="P5" s="110" t="inlineStr">
-        <is>
-          <t>r.prior_loss.p</t>
-        </is>
-      </c>
-      <c r="Q5" s="110" t="inlineStr">
+      <c r="P5" s="555" t="inlineStr">
+        <is>
+          <t>rep_loss.prior</t>
+        </is>
+      </c>
+      <c r="Q5" s="555" t="inlineStr">
         <is>
           <t>pd_loss.prior</t>
         </is>
       </c>
-      <c r="R5" s="110" t="inlineStr">
+      <c r="R5" s="555" t="inlineStr">
         <is>
           <t>case_loss.prior</t>
         </is>
       </c>
-      <c r="S5" s="110" t="inlineStr">
-        <is>
-          <t>sou.currente.prior</t>
-        </is>
-      </c>
-      <c r="T5" s="110"/>
+      <c r="S5" s="564" t="inlineStr">
+        <is>
+          <t>source.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="555"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B6" s="108" t="inlineStr">
-        <is>
-          <t>A0007</t>
-        </is>
-      </c>
-      <c r="C6" s="114">
-        <v>44064</v>
-      </c>
-      <c r="D6" s="114">
-        <v>44745</v>
-      </c>
-      <c r="E6" s="114">
-        <v>44757</v>
-      </c>
-      <c r="F6" s="108" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="G6" s="108">
-        <v>7843</v>
-      </c>
-      <c r="H6" s="108">
-        <v>7843</v>
-      </c>
-      <c r="I6" s="108">
-        <v>0</v>
-      </c>
-      <c r="J6" s="108" t="inlineStr">
-        <is>
-          <t>ex1_curr</t>
-        </is>
-      </c>
-      <c r="K6" s="108" t="inlineStr">
-        <is>
-          <t>A0007</t>
-        </is>
-      </c>
-      <c r="L6" s="118">
-        <v>44054</v>
-      </c>
-      <c r="M6" s="118">
-        <v>44745</v>
-      </c>
-      <c r="N6" s="118">
-        <v>44757</v>
-      </c>
-      <c r="O6" s="108" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="P6" s="108">
-        <v>7843</v>
-      </c>
-      <c r="Q6" s="108">
-        <v>7843</v>
-      </c>
-      <c r="R6" s="108">
-        <v>0</v>
-      </c>
-      <c r="S6" s="108" t="inlineStr">
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B6" s="565" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6" s="559" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D6" s="559" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E6" s="559" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="553" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6" s="553" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" s="553" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" s="553" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" s="565" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K6" s="565" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="L6" s="563">
+        <v>44312</v>
+      </c>
+      <c r="M6" s="563">
+        <v>44545</v>
+      </c>
+      <c r="N6" s="563" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="553" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P6" s="553">
+        <v>17378</v>
+      </c>
+      <c r="Q6" s="553">
+        <v>12512</v>
+      </c>
+      <c r="R6" s="553">
+        <v>4866</v>
+      </c>
+      <c r="S6" s="565" t="inlineStr">
         <is>
           <t>ex1_prior</t>
         </is>
       </c>
-      <c r="T6" s="108"/>
+      <c r="T6" s="553"/>
     </row>
     <row r="7">
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="L7" s="116"/>
-      <c r="M7" s="116"/>
-      <c r="N7" s="116"/>
+      <c r="B7" s="210"/>
+      <c r="C7" s="557"/>
+      <c r="D7" s="557"/>
+      <c r="E7" s="557"/>
+      <c r="J7" s="210"/>
+      <c r="K7" s="210"/>
+      <c r="L7" s="561"/>
+      <c r="M7" s="561"/>
+      <c r="N7" s="561"/>
+      <c r="S7" s="210"/>
     </row>
     <row r="8">
-      <c r="C8" s="112"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="L8" s="116"/>
-      <c r="M8" s="116"/>
-      <c r="N8" s="116"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="557"/>
+      <c r="D8" s="557"/>
+      <c r="E8" s="557"/>
+      <c r="J8" s="210"/>
+      <c r="K8" s="210"/>
+      <c r="L8" s="561"/>
+      <c r="M8" s="561"/>
+      <c r="N8" s="561"/>
+      <c r="S8" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -1988,7 +2949,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -1997,255 +2958,457 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>claim number disappeared</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="122"/>
+          <t>retroactive changes</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="579"/>
+      <c r="D1" s="579"/>
+      <c r="E1" s="579"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="126"/>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="219"/>
+      <c r="L1" s="583"/>
+      <c r="M1" s="583"/>
+      <c r="N1" s="583"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
+      <c r="S1" s="219"/>
       <c r="T1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, rolling time window, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="123"/>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
-      <c r="L2" s="127"/>
-      <c r="M2" s="127"/>
-      <c r="N2" s="127"/>
+          <t>could be timing issues, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="580"/>
+      <c r="D2" s="580"/>
+      <c r="E2" s="580"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="584"/>
+      <c r="M2" s="584"/>
+      <c r="N2" s="584"/>
+      <c r="S2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="L3" s="127"/>
-      <c r="M3" s="127"/>
-      <c r="N3" s="127"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="580"/>
+      <c r="D3" s="580"/>
+      <c r="E3" s="580"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="584"/>
+      <c r="M3" s="584"/>
+      <c r="N3" s="584"/>
+      <c r="S3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="123"/>
-      <c r="D4" s="123"/>
-      <c r="E4" s="123"/>
-      <c r="L4" s="127"/>
-      <c r="M4" s="127"/>
-      <c r="N4" s="127"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="580"/>
+      <c r="D4" s="580"/>
+      <c r="E4" s="580"/>
+      <c r="J4" s="210"/>
+      <c r="K4" s="210"/>
+      <c r="L4" s="584"/>
+      <c r="M4" s="584"/>
+      <c r="N4" s="584"/>
+      <c r="S4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="121" t="inlineStr">
+      <c r="B5" s="577" t="inlineStr">
         <is>
           <t>claim_num.current</t>
         </is>
       </c>
-      <c r="C5" s="124" t="inlineStr">
-        <is>
-          <t>.currentc_date.c</t>
-        </is>
-      </c>
-      <c r="D5" s="124" t="inlineStr">
-        <is>
-          <t>r.prior_date.current</t>
-        </is>
-      </c>
-      <c r="E5" s="124" t="inlineStr">
+      <c r="C5" s="581" t="inlineStr">
+        <is>
+          <t>acc_date.current</t>
+        </is>
+      </c>
+      <c r="D5" s="581" t="inlineStr">
+        <is>
+          <t>rep_date.current</t>
+        </is>
+      </c>
+      <c r="E5" s="581" t="inlineStr">
         <is>
           <t>clsd_date.current</t>
         </is>
       </c>
-      <c r="F5" s="121" t="inlineStr">
+      <c r="F5" s="568" t="inlineStr">
         <is>
           <t>claim_status.current</t>
         </is>
       </c>
-      <c r="G5" s="121" t="inlineStr">
-        <is>
-          <t>r.prior_loss.current</t>
-        </is>
-      </c>
-      <c r="H5" s="121" t="inlineStr">
+      <c r="G5" s="568" t="inlineStr">
+        <is>
+          <t>rep_loss.current</t>
+        </is>
+      </c>
+      <c r="H5" s="568" t="inlineStr">
         <is>
           <t>pd_loss.current</t>
         </is>
       </c>
-      <c r="I5" s="121" t="inlineStr">
+      <c r="I5" s="568" t="inlineStr">
         <is>
           <t>case_loss.current</t>
         </is>
       </c>
-      <c r="J5" s="121" t="inlineStr">
-        <is>
-          <t>sou.currente.c</t>
-        </is>
-      </c>
-      <c r="K5" s="121" t="inlineStr">
+      <c r="J5" s="577" t="inlineStr">
+        <is>
+          <t>source.current</t>
+        </is>
+      </c>
+      <c r="K5" s="577" t="inlineStr">
         <is>
           <t>claim_num.prior</t>
         </is>
       </c>
-      <c r="L5" s="128" t="inlineStr">
-        <is>
-          <t>.currentc_date.prior</t>
-        </is>
-      </c>
-      <c r="M5" s="128" t="inlineStr">
-        <is>
-          <t>r.prior_date.p</t>
-        </is>
-      </c>
-      <c r="N5" s="128" t="inlineStr">
+      <c r="L5" s="585" t="inlineStr">
+        <is>
+          <t>acc_date.prior</t>
+        </is>
+      </c>
+      <c r="M5" s="585" t="inlineStr">
+        <is>
+          <t>rep_date.prior</t>
+        </is>
+      </c>
+      <c r="N5" s="585" t="inlineStr">
         <is>
           <t>clsd_date.prior</t>
         </is>
       </c>
-      <c r="O5" s="121" t="inlineStr">
+      <c r="O5" s="568" t="inlineStr">
         <is>
           <t>claim_status.prior</t>
         </is>
       </c>
-      <c r="P5" s="121" t="inlineStr">
-        <is>
-          <t>r.prior_loss.p</t>
-        </is>
-      </c>
-      <c r="Q5" s="121" t="inlineStr">
+      <c r="P5" s="568" t="inlineStr">
+        <is>
+          <t>rep_loss.prior</t>
+        </is>
+      </c>
+      <c r="Q5" s="568" t="inlineStr">
         <is>
           <t>pd_loss.prior</t>
         </is>
       </c>
-      <c r="R5" s="121" t="inlineStr">
+      <c r="R5" s="568" t="inlineStr">
         <is>
           <t>case_loss.prior</t>
         </is>
       </c>
-      <c r="S5" s="121" t="inlineStr">
-        <is>
-          <t>sou.currente.prior</t>
-        </is>
-      </c>
-      <c r="T5" s="121"/>
+      <c r="S5" s="577" t="inlineStr">
+        <is>
+          <t>source.prior</t>
+        </is>
+      </c>
+      <c r="T5" s="568"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C6" s="125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D6" s="125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E6" s="125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J6" s="119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K6" s="119" t="inlineStr">
-        <is>
-          <t>A0010</t>
-        </is>
-      </c>
-      <c r="L6" s="129">
-        <v>44312</v>
-      </c>
-      <c r="M6" s="129">
-        <v>44545</v>
-      </c>
-      <c r="N6" s="129" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O6" s="119" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="P6" s="119">
-        <v>17378</v>
-      </c>
-      <c r="Q6" s="119">
-        <v>12512</v>
-      </c>
-      <c r="R6" s="119">
-        <v>4866</v>
-      </c>
-      <c r="S6" s="119" t="inlineStr">
-        <is>
-          <t>ex1_prior</t>
-        </is>
-      </c>
-      <c r="T6" s="119"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" s="578" t="inlineStr">
+        <is>
+          <t>A0011</t>
+        </is>
+      </c>
+      <c r="C6" s="582">
+        <v>44330</v>
+      </c>
+      <c r="D6" s="582">
+        <v>44853</v>
+      </c>
+      <c r="E6" s="582">
+        <v>44897</v>
+      </c>
+      <c r="F6" s="566" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="566">
+        <v>62968</v>
+      </c>
+      <c r="H6" s="566">
+        <v>61968</v>
+      </c>
+      <c r="I6" s="566">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="578" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K6" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N6" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P6" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q6" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R6" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S6" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" s="566"/>
     </row>
     <row r="7">
-      <c r="C7" s="123"/>
-      <c r="D7" s="123"/>
-      <c r="E7" s="123"/>
-      <c r="L7" s="127"/>
-      <c r="M7" s="127"/>
-      <c r="N7" s="127"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B7" s="578" t="inlineStr">
+        <is>
+          <t>A0012</t>
+        </is>
+      </c>
+      <c r="C7" s="582">
+        <v>44302</v>
+      </c>
+      <c r="D7" s="582">
+        <v>44354</v>
+      </c>
+      <c r="E7" s="582">
+        <v>44641</v>
+      </c>
+      <c r="F7" s="566" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G7" s="566">
+        <v>44128</v>
+      </c>
+      <c r="H7" s="566">
+        <v>44128</v>
+      </c>
+      <c r="I7" s="566">
+        <v>0</v>
+      </c>
+      <c r="J7" s="578" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="K7" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M7" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N7" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P7" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q7" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R7" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S7" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T7" s="566"/>
     </row>
     <row r="8">
-      <c r="C8" s="123"/>
-      <c r="D8" s="123"/>
-      <c r="E8" s="123"/>
-      <c r="L8" s="127"/>
-      <c r="M8" s="127"/>
-      <c r="N8" s="127"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="B8" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" s="582" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D8" s="582" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E8" s="582" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" s="586" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" s="566" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S8" s="578" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" s="566"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="210"/>
+      <c r="C9" s="580"/>
+      <c r="D9" s="580"/>
+      <c r="E9" s="580"/>
+      <c r="J9" s="210"/>
+      <c r="K9" s="210"/>
+      <c r="L9" s="584"/>
+      <c r="M9" s="584"/>
+      <c r="N9" s="584"/>
+      <c r="S9" s="210"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="210"/>
+      <c r="C10" s="580"/>
+      <c r="D10" s="580"/>
+      <c r="E10" s="580"/>
+      <c r="J10" s="210"/>
+      <c r="K10" s="210"/>
+      <c r="L10" s="584"/>
+      <c r="M10" s="584"/>
+      <c r="N10" s="584"/>
+      <c r="S10" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -2285,22 +3448,22 @@
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="131" t="inlineStr">
+      <c r="B5" s="588" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="C5" s="131" t="inlineStr">
+      <c r="C5" s="588" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="D5" s="131" t="inlineStr">
+      <c r="D5" s="588" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="E5" s="131"/>
+      <c r="E5" s="588"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2308,20 +3471,20 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B6" s="130" t="inlineStr">
+      <c r="B6" s="587" t="inlineStr">
         <is>
           <t>maybe missing claims</t>
         </is>
       </c>
-      <c r="C6" s="130" t="inlineStr">
+      <c r="C6" s="587" t="inlineStr">
         <is>
           <t>claim numbers which potentially should show up but don't</t>
         </is>
       </c>
-      <c r="D6" s="130">
+      <c r="D6" s="587">
         <v>1</v>
       </c>
-      <c r="E6" s="130"/>
+      <c r="E6" s="587"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2329,20 +3492,20 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B7" s="130" t="inlineStr">
+      <c r="B7" s="587" t="inlineStr">
         <is>
           <t>claim dupes</t>
         </is>
       </c>
-      <c r="C7" s="130" t="inlineStr">
+      <c r="C7" s="587" t="inlineStr">
         <is>
           <t>claim numbers which show up multiple times</t>
         </is>
       </c>
-      <c r="D7" s="130">
+      <c r="D7" s="587">
         <v>0</v>
       </c>
-      <c r="E7" s="130"/>
+      <c r="E7" s="587"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2350,20 +3513,20 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B8" s="130" t="inlineStr">
+      <c r="B8" s="587" t="inlineStr">
         <is>
           <t>closure flag vs case</t>
         </is>
       </c>
-      <c r="C8" s="130" t="inlineStr">
+      <c r="C8" s="587" t="inlineStr">
         <is>
           <t>closure flag which doesn't seem to match case reserves</t>
         </is>
       </c>
-      <c r="D8" s="130">
+      <c r="D8" s="587">
         <v>1</v>
       </c>
-      <c r="E8" s="130"/>
+      <c r="E8" s="587"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2371,20 +3534,20 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B9" s="130" t="inlineStr">
+      <c r="B9" s="587" t="inlineStr">
         <is>
           <t>closure flag vs close date</t>
         </is>
       </c>
-      <c r="C9" s="130" t="inlineStr">
+      <c r="C9" s="587" t="inlineStr">
         <is>
           <t>closure flag which doesn't seem to match close date</t>
         </is>
       </c>
-      <c r="D9" s="130">
+      <c r="D9" s="587">
         <v>0</v>
       </c>
-      <c r="E9" s="130"/>
+      <c r="E9" s="587"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -2392,20 +3555,20 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B10" s="130" t="inlineStr">
+      <c r="B10" s="587" t="inlineStr">
         <is>
           <t>close date &lt; report date</t>
         </is>
       </c>
-      <c r="C10" s="130" t="inlineStr">
+      <c r="C10" s="587" t="inlineStr">
         <is>
           <t>close date &lt; report date</t>
         </is>
       </c>
-      <c r="D10" s="130">
+      <c r="D10" s="587">
         <v>0</v>
       </c>
-      <c r="E10" s="130"/>
+      <c r="E10" s="587"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2413,20 +3576,20 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B11" s="130" t="inlineStr">
+      <c r="B11" s="587" t="inlineStr">
         <is>
           <t>report date &lt; loss date</t>
         </is>
       </c>
-      <c r="C11" s="130" t="inlineStr">
+      <c r="C11" s="587" t="inlineStr">
         <is>
           <t>report date &lt; loss date</t>
         </is>
       </c>
-      <c r="D11" s="130">
+      <c r="D11" s="587">
         <v>0</v>
       </c>
-      <c r="E11" s="130"/>
+      <c r="E11" s="587"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2434,20 +3597,20 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B12" s="130" t="inlineStr">
+      <c r="B12" s="587" t="inlineStr">
         <is>
           <t>missing loss or report date</t>
         </is>
       </c>
-      <c r="C12" s="130" t="inlineStr">
+      <c r="C12" s="587" t="inlineStr">
         <is>
           <t>missing loss or report date</t>
         </is>
       </c>
-      <c r="D12" s="130">
+      <c r="D12" s="587">
         <v>0</v>
       </c>
-      <c r="E12" s="130"/>
+      <c r="E12" s="587"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -2455,20 +3618,20 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B13" s="130" t="inlineStr">
+      <c r="B13" s="587" t="inlineStr">
         <is>
           <t>negative paid or case</t>
         </is>
       </c>
-      <c r="C13" s="130" t="inlineStr">
+      <c r="C13" s="587" t="inlineStr">
         <is>
           <t>negative paid or case</t>
         </is>
       </c>
-      <c r="D13" s="130">
+      <c r="D13" s="587">
         <v>0</v>
       </c>
-      <c r="E13" s="130"/>
+      <c r="E13" s="587"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -2476,20 +3639,20 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B14" s="130" t="inlineStr">
+      <c r="B14" s="587" t="inlineStr">
         <is>
           <t>paid+case vs rptd</t>
         </is>
       </c>
-      <c r="C14" s="130" t="inlineStr">
+      <c r="C14" s="587" t="inlineStr">
         <is>
           <t>paid+case vs rptd</t>
         </is>
       </c>
-      <c r="D14" s="130">
+      <c r="D14" s="587">
         <v>1</v>
       </c>
-      <c r="E14" s="130"/>
+      <c r="E14" s="587"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -2497,20 +3660,20 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B15" s="130" t="inlineStr">
+      <c r="B15" s="587" t="inlineStr">
         <is>
           <t>paid decreased</t>
         </is>
       </c>
-      <c r="C15" s="130" t="inlineStr">
+      <c r="C15" s="587" t="inlineStr">
         <is>
           <t>paid decreased</t>
         </is>
       </c>
-      <c r="D15" s="130">
+      <c r="D15" s="587">
         <v>2</v>
       </c>
-      <c r="E15" s="130"/>
+      <c r="E15" s="587"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -2518,20 +3681,20 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B16" s="130" t="inlineStr">
+      <c r="B16" s="587" t="inlineStr">
         <is>
           <t>date decreased</t>
         </is>
       </c>
-      <c r="C16" s="130" t="inlineStr">
+      <c r="C16" s="587" t="inlineStr">
         <is>
           <t>loss/report date decreased or disappeared</t>
         </is>
       </c>
-      <c r="D16" s="130">
+      <c r="D16" s="587">
         <v>0</v>
       </c>
-      <c r="E16" s="130"/>
+      <c r="E16" s="587"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2539,20 +3702,20 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B17" s="130" t="inlineStr">
+      <c r="B17" s="587" t="inlineStr">
         <is>
           <t>loss or report date changed</t>
         </is>
       </c>
-      <c r="C17" s="130" t="inlineStr">
+      <c r="C17" s="587" t="inlineStr">
         <is>
           <t>loss or report date changed</t>
         </is>
       </c>
-      <c r="D17" s="130">
+      <c r="D17" s="587">
         <v>1</v>
       </c>
-      <c r="E17" s="130"/>
+      <c r="E17" s="587"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -2560,20 +3723,20 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B18" s="130" t="inlineStr">
+      <c r="B18" s="587" t="inlineStr">
         <is>
           <t>claim number disappeared</t>
         </is>
       </c>
-      <c r="C18" s="130" t="inlineStr">
+      <c r="C18" s="587" t="inlineStr">
         <is>
           <t>claim number present in prior but not current</t>
         </is>
       </c>
-      <c r="D18" s="130">
+      <c r="D18" s="587">
         <v>1</v>
       </c>
-      <c r="E18" s="130"/>
+      <c r="E18" s="587"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2581,20 +3744,20 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B19" s="130" t="inlineStr">
+      <c r="B19" s="587" t="inlineStr">
         <is>
           <t>did we get new claims since last time?</t>
         </is>
       </c>
-      <c r="C19" s="130" t="inlineStr">
+      <c r="C19" s="587" t="inlineStr">
         <is>
           <t>1 if we got no new claims since prior loss run, else 0</t>
         </is>
       </c>
-      <c r="D19" s="130">
+      <c r="D19" s="587">
         <v>0</v>
       </c>
-      <c r="E19" s="130"/>
+      <c r="E19" s="587"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -2602,20 +3765,20 @@
           <t>15</t>
         </is>
       </c>
-      <c r="B20" s="130" t="inlineStr">
+      <c r="B20" s="587" t="inlineStr">
         <is>
           <t>retroactive changes</t>
         </is>
       </c>
-      <c r="C20" s="130" t="inlineStr">
+      <c r="C20" s="587" t="inlineStr">
         <is>
           <t>new claims added in current loss run, with loss/report/close date likely prior to the evaluation date of the prior loss run</t>
         </is>
       </c>
-      <c r="D20" s="130">
-        <v>0</v>
-      </c>
-      <c r="E20" s="130"/>
+      <c r="D20" s="587">
+        <v>3</v>
+      </c>
+      <c r="E20" s="587"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -5328,176 +6491,86 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="20" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>retroactive changes</t>
+          <t>maybe missing claims</t>
         </is>
       </c>
       <c r="B1" s="7"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
+      <c r="C1" s="493"/>
+      <c r="D1" s="493"/>
+      <c r="E1" s="494"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be timing issues, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
+          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
+        </is>
+      </c>
+      <c r="C2" s="494"/>
+      <c r="D2" s="494"/>
+      <c r="E2" s="494"/>
     </row>
     <row r="3">
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="L3" s="73"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="73"/>
+      <c r="C3" s="494"/>
+      <c r="D3" s="494"/>
+      <c r="E3" s="494"/>
     </row>
     <row r="4">
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
+      <c r="C4" s="494"/>
+      <c r="D4" s="494"/>
+      <c r="E4" s="494"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="68" t="inlineStr">
-        <is>
-          <t>claim_num.c</t>
-        </is>
-      </c>
-      <c r="C5" s="71" t="inlineStr">
-        <is>
-          <t>acc_date.c</t>
-        </is>
-      </c>
-      <c r="D5" s="71" t="inlineStr">
-        <is>
-          <t>rep_date.c</t>
-        </is>
-      </c>
-      <c r="E5" s="71" t="inlineStr">
-        <is>
-          <t>clsd_date.c</t>
-        </is>
-      </c>
-      <c r="F5" s="68" t="inlineStr">
-        <is>
-          <t>claim_status.c</t>
-        </is>
-      </c>
-      <c r="G5" s="68" t="inlineStr">
-        <is>
-          <t>rep_loss.c</t>
-        </is>
-      </c>
-      <c r="H5" s="68" t="inlineStr">
-        <is>
-          <t>pd_loss.c</t>
-        </is>
-      </c>
-      <c r="I5" s="68" t="inlineStr">
-        <is>
-          <t>case_loss.c</t>
-        </is>
-      </c>
-      <c r="J5" s="68" t="inlineStr">
-        <is>
-          <t>source.c</t>
-        </is>
-      </c>
-      <c r="K5" s="68" t="inlineStr">
-        <is>
-          <t>claim_num.p</t>
-        </is>
-      </c>
-      <c r="L5" s="74" t="inlineStr">
-        <is>
-          <t>acc_date.p</t>
-        </is>
-      </c>
-      <c r="M5" s="74" t="inlineStr">
-        <is>
-          <t>rep_date.p</t>
-        </is>
-      </c>
-      <c r="N5" s="74" t="inlineStr">
-        <is>
-          <t>clsd_date.p</t>
-        </is>
-      </c>
-      <c r="O5" s="68" t="inlineStr">
-        <is>
-          <t>claim_status.p</t>
-        </is>
-      </c>
-      <c r="P5" s="68" t="inlineStr">
-        <is>
-          <t>rep_loss.p</t>
-        </is>
-      </c>
-      <c r="Q5" s="68" t="inlineStr">
-        <is>
-          <t>pd_loss.p</t>
-        </is>
-      </c>
-      <c r="R5" s="68" t="inlineStr">
-        <is>
-          <t>case_loss.p</t>
-        </is>
-      </c>
-      <c r="S5" s="68" t="inlineStr">
-        <is>
-          <t>source.p</t>
-        </is>
-      </c>
-      <c r="T5" s="68"/>
+      <c r="B5" s="492" t="inlineStr">
+        <is>
+          <t>claim_num.x</t>
+        </is>
+      </c>
+      <c r="C5" s="495" t="inlineStr">
+        <is>
+          <t>source.x</t>
+        </is>
+      </c>
+      <c r="D5" s="495"/>
+      <c r="E5" s="494"/>
     </row>
     <row r="6">
-      <c r="C6" s="70"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="L6" s="73"/>
-      <c r="M6" s="73"/>
-      <c r="N6" s="73"/>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" s="491" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="C6" s="496" t="inlineStr">
+        <is>
+          <t>ex1_curr</t>
+        </is>
+      </c>
+      <c r="D6" s="496"/>
+      <c r="E6" s="494"/>
     </row>
     <row r="7">
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="L7" s="73"/>
-      <c r="M7" s="73"/>
-      <c r="N7" s="73"/>
+      <c r="C7" s="494"/>
+      <c r="D7" s="494"/>
+      <c r="E7" s="494"/>
+    </row>
+    <row r="8">
+      <c r="C8" s="494"/>
+      <c r="D8" s="494"/>
+      <c r="E8" s="494"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>
@@ -5511,57 +6584,115 @@
   <sheetPr>
     <tabColor rgb="FFFFC0CB"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="1" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>maybe missing claims</t>
-        </is>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="80"/>
+          <t>closure flag vs case</t>
+        </is>
+      </c>
+      <c r="B1" s="219"/>
+      <c r="C1" s="500"/>
+      <c r="D1" s="500"/>
+      <c r="E1" s="506"/>
+      <c r="F1" s="219"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="219"/>
+      <c r="J1" s="219"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>could be non-sequential claim numbers, CWP/dormant claims removed, portfolio/segmentation change, error correction, something else</t>
-        </is>
-      </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
+          <t>could be something about claims process, timing issue, closure being defined at a different level of aggregation than the claim, something else</t>
+        </is>
+      </c>
+      <c r="B2" s="210"/>
+      <c r="C2" s="501"/>
+      <c r="D2" s="501"/>
+      <c r="E2" s="507"/>
+      <c r="F2" s="210"/>
+      <c r="I2" s="210"/>
+      <c r="J2" s="210"/>
     </row>
     <row r="3">
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
+      <c r="B3" s="210"/>
+      <c r="C3" s="501"/>
+      <c r="D3" s="501"/>
+      <c r="E3" s="507"/>
+      <c r="F3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
     </row>
     <row r="4">
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
+      <c r="B4" s="210"/>
+      <c r="C4" s="501"/>
+      <c r="D4" s="501"/>
+      <c r="E4" s="507"/>
+      <c r="F4" s="210"/>
+      <c r="I4" s="210"/>
+      <c r="J4" s="210"/>
     </row>
     <row r="5">
       <c r="A5" s="7"/>
-      <c r="B5" s="78" t="inlineStr">
-        <is>
-          <t>claim_num.x</t>
-        </is>
-      </c>
-      <c r="C5" s="81" t="inlineStr">
-        <is>
-          <t>source.x</t>
-        </is>
-      </c>
-      <c r="D5" s="81"/>
-      <c r="E5" s="80"/>
+      <c r="B5" s="504" t="inlineStr">
+        <is>
+          <t>claim_num</t>
+        </is>
+      </c>
+      <c r="C5" s="502" t="inlineStr">
+        <is>
+          <t>acc_date</t>
+        </is>
+      </c>
+      <c r="D5" s="502" t="inlineStr">
+        <is>
+          <t>rep_date</t>
+        </is>
+      </c>
+      <c r="E5" s="508" t="inlineStr">
+        <is>
+          <t>clsd_date</t>
+        </is>
+      </c>
+      <c r="F5" s="504" t="inlineStr">
+        <is>
+          <t>claim_status</t>
+        </is>
+      </c>
+      <c r="G5" s="499" t="inlineStr">
+        <is>
+          <t>rep_loss</t>
+        </is>
+      </c>
+      <c r="H5" s="499" t="inlineStr">
+        <is>
+          <t>pd_loss</t>
+        </is>
+      </c>
+      <c r="I5" s="504" t="inlineStr">
+        <is>
+          <t>case_loss</t>
+        </is>
+      </c>
+      <c r="J5" s="504" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="499" t="inlineStr">
+        <is>
+          <t>zero_case</t>
+        </is>
+      </c>
+      <c r="L5" s="499"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -5569,28 +6700,61 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B6" s="77" t="inlineStr">
-        <is>
-          <t>A0010</t>
-        </is>
-      </c>
-      <c r="C6" s="82" t="inlineStr">
+      <c r="B6" s="505" t="inlineStr">
+        <is>
+          <t>A0011</t>
+        </is>
+      </c>
+      <c r="C6" s="503">
+        <v>44330</v>
+      </c>
+      <c r="D6" s="503">
+        <v>44853</v>
+      </c>
+      <c r="E6" s="509">
+        <v>44897</v>
+      </c>
+      <c r="F6" s="505" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G6" s="497">
+        <v>62968</v>
+      </c>
+      <c r="H6" s="497">
+        <v>61968</v>
+      </c>
+      <c r="I6" s="505">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="505" t="inlineStr">
         <is>
           <t>ex1_curr</t>
         </is>
       </c>
-      <c r="D6" s="82"/>
-      <c r="E6" s="80"/>
+      <c r="K6" s="497" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="497"/>
     </row>
     <row r="7">
-      <c r="C7" s="80"/>
-      <c r="D7" s="80"/>
-      <c r="E7" s="80"/>
+      <c r="B7" s="210"/>
+      <c r="C7" s="501"/>
+      <c r="D7" s="501"/>
+      <c r="E7" s="507"/>
+      <c r="F7" s="210"/>
+      <c r="I7" s="210"/>
+      <c r="J7" s="210"/>
     </row>
     <row r="8">
-      <c r="C8" s="80"/>
-      <c r="D8" s="80"/>
-      <c r="E8" s="80"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="501"/>
+      <c r="D8" s="501"/>
+      <c r="E8" s="507"/>
+      <c r="F8" s="210"/>
+      <c r="I8" s="210"/>
+      <c r="J8" s="210"/>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>

</xml_diff>